<commit_message>
Implemented mass balance calculations for manure N,P,K excretion
</commit_message>
<xml_diff>
--- a/data/default/CattleHerd.xlsx
+++ b/data/default/CattleHerd.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\prod_parameters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19020" windowHeight="6705" tabRatio="846" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19020" windowHeight="6705" tabRatio="846" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="13" r:id="rId1"/>
@@ -3307,12 +3307,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="40" fillId="41" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3324,6 +3318,12 @@
     </xf>
     <xf numFmtId="0" fontId="40" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -36050,49 +36050,49 @@
       </c>
       <c r="AB3" s="202"/>
       <c r="AC3" s="202"/>
-      <c r="AD3" s="261" t="s">
+      <c r="AD3" s="259" t="s">
         <v>543</v>
       </c>
-      <c r="AE3" s="262" t="s">
+      <c r="AE3" s="260" t="s">
         <v>545</v>
       </c>
-      <c r="AF3" s="261" t="s">
+      <c r="AF3" s="259" t="s">
         <v>547</v>
       </c>
-      <c r="AG3" s="262" t="s">
+      <c r="AG3" s="260" t="s">
         <v>549</v>
       </c>
-      <c r="AH3" s="261" t="s">
+      <c r="AH3" s="259" t="s">
         <v>550</v>
       </c>
-      <c r="AI3" s="262" t="s">
+      <c r="AI3" s="260" t="s">
         <v>552</v>
       </c>
-      <c r="AJ3" s="261" t="s">
+      <c r="AJ3" s="259" t="s">
         <v>553</v>
       </c>
-      <c r="AK3" s="262" t="s">
+      <c r="AK3" s="260" t="s">
         <v>554</v>
       </c>
-      <c r="AL3" s="261" t="s">
+      <c r="AL3" s="259" t="s">
         <v>556</v>
       </c>
-      <c r="AM3" s="262" t="s">
+      <c r="AM3" s="260" t="s">
         <v>557</v>
       </c>
-      <c r="AN3" s="261" t="s">
+      <c r="AN3" s="259" t="s">
         <v>577</v>
       </c>
-      <c r="AO3" s="262" t="s">
+      <c r="AO3" s="260" t="s">
         <v>559</v>
       </c>
-      <c r="AP3" s="261" t="s">
+      <c r="AP3" s="259" t="s">
         <v>560</v>
       </c>
-      <c r="AQ3" s="260" t="s">
+      <c r="AQ3" s="258" t="s">
         <v>581</v>
       </c>
-      <c r="AR3" s="259" t="s">
+      <c r="AR3" s="257" t="s">
         <v>576</v>
       </c>
     </row>
@@ -36143,21 +36143,21 @@
       <c r="AA4" s="201"/>
       <c r="AB4" s="202"/>
       <c r="AC4" s="202"/>
-      <c r="AD4" s="261"/>
-      <c r="AE4" s="262"/>
-      <c r="AF4" s="261"/>
-      <c r="AG4" s="262"/>
-      <c r="AH4" s="261"/>
-      <c r="AI4" s="262"/>
-      <c r="AJ4" s="261"/>
-      <c r="AK4" s="262"/>
-      <c r="AL4" s="261"/>
-      <c r="AM4" s="262"/>
-      <c r="AN4" s="261"/>
-      <c r="AO4" s="262"/>
-      <c r="AP4" s="261"/>
-      <c r="AQ4" s="260"/>
-      <c r="AR4" s="259"/>
+      <c r="AD4" s="259"/>
+      <c r="AE4" s="260"/>
+      <c r="AF4" s="259"/>
+      <c r="AG4" s="260"/>
+      <c r="AH4" s="259"/>
+      <c r="AI4" s="260"/>
+      <c r="AJ4" s="259"/>
+      <c r="AK4" s="260"/>
+      <c r="AL4" s="259"/>
+      <c r="AM4" s="260"/>
+      <c r="AN4" s="259"/>
+      <c r="AO4" s="260"/>
+      <c r="AP4" s="259"/>
+      <c r="AQ4" s="258"/>
+      <c r="AR4" s="257"/>
     </row>
     <row r="5" spans="2:44" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="209" t="s">
@@ -36238,21 +36238,21 @@
       <c r="AA5" s="201"/>
       <c r="AB5" s="202"/>
       <c r="AC5" s="202"/>
-      <c r="AD5" s="261"/>
-      <c r="AE5" s="262"/>
-      <c r="AF5" s="261"/>
-      <c r="AG5" s="262"/>
-      <c r="AH5" s="261"/>
-      <c r="AI5" s="262"/>
-      <c r="AJ5" s="261"/>
-      <c r="AK5" s="262"/>
-      <c r="AL5" s="261"/>
-      <c r="AM5" s="262"/>
-      <c r="AN5" s="261"/>
-      <c r="AO5" s="262"/>
-      <c r="AP5" s="261"/>
-      <c r="AQ5" s="260"/>
-      <c r="AR5" s="259" t="s">
+      <c r="AD5" s="259"/>
+      <c r="AE5" s="260"/>
+      <c r="AF5" s="259"/>
+      <c r="AG5" s="260"/>
+      <c r="AH5" s="259"/>
+      <c r="AI5" s="260"/>
+      <c r="AJ5" s="259"/>
+      <c r="AK5" s="260"/>
+      <c r="AL5" s="259"/>
+      <c r="AM5" s="260"/>
+      <c r="AN5" s="259"/>
+      <c r="AO5" s="260"/>
+      <c r="AP5" s="259"/>
+      <c r="AQ5" s="258"/>
+      <c r="AR5" s="257" t="s">
         <v>575</v>
       </c>
     </row>
@@ -37687,23 +37687,23 @@
       <c r="N23" s="169"/>
       <c r="O23" s="169"/>
       <c r="P23" s="169"/>
-      <c r="Q23" s="258" t="s">
+      <c r="Q23" s="262" t="s">
         <v>596</v>
       </c>
-      <c r="R23" s="258" t="s">
+      <c r="R23" s="262" t="s">
         <v>597</v>
       </c>
-      <c r="S23" s="258" t="s">
+      <c r="S23" s="262" t="s">
         <v>584</v>
       </c>
-      <c r="T23" s="257" t="s">
+      <c r="T23" s="261" t="s">
         <v>303</v>
       </c>
-      <c r="U23" s="257"/>
-      <c r="V23" s="257" t="s">
+      <c r="U23" s="261"/>
+      <c r="V23" s="261" t="s">
         <v>304</v>
       </c>
-      <c r="W23" s="257"/>
+      <c r="W23" s="261"/>
       <c r="X23" s="168" t="s">
         <v>482</v>
       </c>
@@ -37728,9 +37728,9 @@
       <c r="P24" s="170" t="s">
         <v>483</v>
       </c>
-      <c r="Q24" s="258"/>
-      <c r="R24" s="258"/>
-      <c r="S24" s="258"/>
+      <c r="Q24" s="262"/>
+      <c r="R24" s="262"/>
+      <c r="S24" s="262"/>
       <c r="T24" s="244" t="s">
         <v>483</v>
       </c>
@@ -44348,6 +44348,11 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="V23:W23"/>
+    <mergeCell ref="T23:U23"/>
+    <mergeCell ref="Q23:Q24"/>
+    <mergeCell ref="R23:R24"/>
+    <mergeCell ref="S23:S24"/>
     <mergeCell ref="AR3:AR5"/>
     <mergeCell ref="AQ3:AQ5"/>
     <mergeCell ref="AD3:AD5"/>
@@ -44363,11 +44368,6 @@
     <mergeCell ref="AN3:AN5"/>
     <mergeCell ref="AO3:AO5"/>
     <mergeCell ref="AP3:AP5"/>
-    <mergeCell ref="V23:W23"/>
-    <mergeCell ref="T23:U23"/>
-    <mergeCell ref="Q23:Q24"/>
-    <mergeCell ref="R23:R24"/>
-    <mergeCell ref="S23:S24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated data: SNG yields, pasture utilisiation, reduced grazing in dairy cow rations, max share SNG of grazing
</commit_message>
<xml_diff>
--- a/data/default/CattleHerd.xlsx
+++ b/data/default/CattleHerd.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18360" windowHeight="6705" tabRatio="846" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18360" windowHeight="6705" tabRatio="846" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="13" r:id="rId1"/>
@@ -144,7 +144,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4205" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4217" uniqueCount="624">
   <si>
     <t>value</t>
   </si>
@@ -1691,9 +1691,6 @@
     <t>Assumes same as dairy cows</t>
   </si>
   <si>
-    <t>Ahlgren et al. (2022) Miljöpåverkan av svensk nöt- och lammköttsproduktion</t>
-  </si>
-  <si>
     <t>Växa Husdjursstatistik 2020, tab 32</t>
   </si>
   <si>
@@ -1995,6 +1992,33 @@
   <si>
     <t>Set to give ~7 kg/calf/day</t>
   </si>
+  <si>
+    <t>Ahlgren, S., Behaderovic, D., Wirsenius, S., Carlsson, A., Hessle, A. Toräng, P., Seeman, A., den Braver, T. &amp;  et al. Kvarnbäck, O. (2022) Miljöpåverkan av svensk nöt- och lammköttsproduktion. RISE</t>
+  </si>
+  <si>
+    <t>Ahlgren et al. (2022)</t>
+  </si>
+  <si>
+    <t>agricultrual statistics</t>
+  </si>
+  <si>
+    <t>grazing factor:</t>
+  </si>
+  <si>
+    <t>ley factor:</t>
+  </si>
+  <si>
+    <t>Grazing share (% of roughage):</t>
+  </si>
+  <si>
+    <t>Grazing factor set to align 'Ley for fodder'</t>
+  </si>
+  <si>
+    <t>Einarsson et al 2022 share grazing of roughage for dairy cows</t>
+  </si>
+  <si>
+    <t>and 'Ley for grazing' areas better to</t>
+  </si>
 </sst>
 </file>
 
@@ -2007,7 +2031,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="45" x14ac:knownFonts="1">
+  <fonts count="47" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2338,8 +2362,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="42">
+  <fills count="43">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2570,6 +2609,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2942,7 +2987,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="267">
+  <cellXfs count="275">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3354,12 +3399,6 @@
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="43"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="40" fillId="41" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3372,6 +3411,26 @@
     <xf numFmtId="0" fontId="40" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="46" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="46" fillId="42" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -15476,17 +15535,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:B3"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B2" s="109" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="109" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>604</v>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>615</v>
       </c>
     </row>
   </sheetData>
@@ -16747,7 +16811,7 @@
         <v>312</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>319</v>
@@ -16837,7 +16901,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="J5" s="111">
         <v>8</v>
@@ -16846,7 +16910,7 @@
         <v>9</v>
       </c>
       <c r="L5" s="93" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="M5" t="s">
         <v>282</v>
@@ -16923,7 +16987,7 @@
         <v>5</v>
       </c>
       <c r="I9" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="J9" s="111">
         <v>8</v>
@@ -16932,7 +16996,7 @@
         <v>9</v>
       </c>
       <c r="L9" s="93" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="M9" t="s">
         <v>282</v>
@@ -17011,7 +17075,7 @@
         <v>41</v>
       </c>
       <c r="L13" s="260" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -17019,7 +17083,7 @@
         <v>38</v>
       </c>
       <c r="I14" s="32" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="J14" s="259">
         <v>0</v>
@@ -17402,7 +17466,7 @@
         <v>7</v>
       </c>
       <c r="M37" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
@@ -18020,7 +18084,7 @@
         <v>10</v>
       </c>
       <c r="M66" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.25">
@@ -18043,7 +18107,7 @@
         <v>22</v>
       </c>
       <c r="M67" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.25">
@@ -18066,7 +18130,7 @@
         <v>24</v>
       </c>
       <c r="M68" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
@@ -18089,7 +18153,7 @@
         <v>22</v>
       </c>
       <c r="M69" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.25">
@@ -18112,7 +18176,7 @@
         <v>24</v>
       </c>
       <c r="M70" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.25">
@@ -18135,7 +18199,7 @@
         <v>28</v>
       </c>
       <c r="M71" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.25">
@@ -18158,7 +18222,7 @@
         <v>24</v>
       </c>
       <c r="M72" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
@@ -18181,7 +18245,7 @@
         <v>28</v>
       </c>
       <c r="M73" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
@@ -18204,7 +18268,7 @@
         <v>24</v>
       </c>
       <c r="M74" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
@@ -18244,7 +18308,7 @@
         <v>10</v>
       </c>
       <c r="M76" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.25">
@@ -18267,7 +18331,7 @@
         <v>22</v>
       </c>
       <c r="M77" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.25">
@@ -18290,7 +18354,7 @@
         <v>39</v>
       </c>
       <c r="M78" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.25">
@@ -18313,7 +18377,7 @@
         <v>22</v>
       </c>
       <c r="M79" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.25">
@@ -18336,7 +18400,7 @@
         <v>39</v>
       </c>
       <c r="M80" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.25">
@@ -18359,7 +18423,7 @@
         <v>28</v>
       </c>
       <c r="M81" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.25">
@@ -18382,7 +18446,7 @@
         <v>39</v>
       </c>
       <c r="M82" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.25">
@@ -18405,7 +18469,7 @@
         <v>28</v>
       </c>
       <c r="M83" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.25">
@@ -18428,7 +18492,7 @@
         <v>39</v>
       </c>
       <c r="M84" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.25">
@@ -19011,7 +19075,7 @@
     </row>
     <row r="118" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A118" s="257" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B118" s="158"/>
       <c r="C118" s="158"/>
@@ -19037,12 +19101,12 @@
       </c>
       <c r="E119" s="110"/>
       <c r="F119" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="G119" s="110"/>
       <c r="H119" s="110"/>
       <c r="I119" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J119" s="110">
         <v>5</v>
@@ -19052,7 +19116,7 @@
       </c>
       <c r="L119" s="110"/>
       <c r="M119" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="120" spans="1:13" x14ac:dyDescent="0.25">
@@ -19066,12 +19130,12 @@
       </c>
       <c r="E120" s="110"/>
       <c r="F120" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="G120" s="110"/>
       <c r="H120" s="110"/>
       <c r="I120" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J120" s="110">
         <v>5.4</v>
@@ -19081,7 +19145,7 @@
       </c>
       <c r="L120" s="110"/>
       <c r="M120" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="121" spans="1:13" x14ac:dyDescent="0.25">
@@ -19095,12 +19159,12 @@
       </c>
       <c r="E121" s="110"/>
       <c r="F121" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="G121" s="110"/>
       <c r="H121" s="110"/>
       <c r="I121" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J121" s="110">
         <v>4.9000000000000004</v>
@@ -19110,7 +19174,7 @@
       </c>
       <c r="L121" s="110"/>
       <c r="M121" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="122" spans="1:13" x14ac:dyDescent="0.25">
@@ -19124,12 +19188,12 @@
       </c>
       <c r="E122" s="110"/>
       <c r="F122" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="G122" s="110"/>
       <c r="H122" s="110"/>
       <c r="I122" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J122" s="110">
         <v>5.0999999999999996</v>
@@ -19139,7 +19203,7 @@
       </c>
       <c r="L122" s="110"/>
       <c r="M122" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="123" spans="1:13" x14ac:dyDescent="0.25">
@@ -19153,12 +19217,12 @@
       </c>
       <c r="E123" s="110"/>
       <c r="F123" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G123" s="110"/>
       <c r="H123" s="110"/>
       <c r="I123" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J123" s="110">
         <v>4.9000000000000004</v>
@@ -19168,7 +19232,7 @@
       </c>
       <c r="L123" s="110"/>
       <c r="M123" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="124" spans="1:13" x14ac:dyDescent="0.25">
@@ -19182,12 +19246,12 @@
       </c>
       <c r="E124" s="110"/>
       <c r="F124" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="G124" s="110"/>
       <c r="H124" s="110"/>
       <c r="I124" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J124" s="110">
         <v>5</v>
@@ -19197,7 +19261,7 @@
       </c>
       <c r="L124" s="110"/>
       <c r="M124" s="110" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="125" spans="1:13" x14ac:dyDescent="0.25">
@@ -19211,12 +19275,12 @@
       </c>
       <c r="E125" s="110"/>
       <c r="F125" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G125" s="110"/>
       <c r="H125" s="110"/>
       <c r="I125" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J125" s="110">
         <v>5</v>
@@ -19226,7 +19290,7 @@
       </c>
       <c r="L125" s="110"/>
       <c r="M125" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="126" spans="1:13" x14ac:dyDescent="0.25">
@@ -19240,12 +19304,12 @@
       </c>
       <c r="E126" s="110"/>
       <c r="F126" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G126" s="110"/>
       <c r="H126" s="110"/>
       <c r="I126" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J126" s="110">
         <v>3.1</v>
@@ -19255,7 +19319,7 @@
       </c>
       <c r="L126" s="110"/>
       <c r="M126" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="127" spans="1:13" x14ac:dyDescent="0.25">
@@ -19280,12 +19344,12 @@
       <c r="D128" s="110"/>
       <c r="E128" s="110"/>
       <c r="F128" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="G128" s="110"/>
       <c r="H128" s="110"/>
       <c r="I128" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J128" s="110">
         <v>6.5</v>
@@ -19294,10 +19358,10 @@
         <v>4</v>
       </c>
       <c r="L128" s="110" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="M128" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="129" spans="1:13" x14ac:dyDescent="0.25">
@@ -19307,12 +19371,12 @@
       <c r="D129" s="110"/>
       <c r="E129" s="110"/>
       <c r="F129" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="G129" s="110"/>
       <c r="H129" s="110"/>
       <c r="I129" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J129" s="110">
         <v>6.8</v>
@@ -19322,7 +19386,7 @@
       </c>
       <c r="L129" s="110"/>
       <c r="M129" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="130" spans="1:13" x14ac:dyDescent="0.25">
@@ -19332,12 +19396,12 @@
       <c r="D130" s="110"/>
       <c r="E130" s="110"/>
       <c r="F130" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="G130" s="110"/>
       <c r="H130" s="110"/>
       <c r="I130" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J130" s="110">
         <v>6.2</v>
@@ -19347,7 +19411,7 @@
       </c>
       <c r="L130" s="110"/>
       <c r="M130" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="131" spans="1:13" x14ac:dyDescent="0.25">
@@ -19357,12 +19421,12 @@
       <c r="D131" s="110"/>
       <c r="E131" s="110"/>
       <c r="F131" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="G131" s="110"/>
       <c r="H131" s="110"/>
       <c r="I131" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J131" s="110">
         <v>6.3</v>
@@ -19372,7 +19436,7 @@
       </c>
       <c r="L131" s="110"/>
       <c r="M131" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="132" spans="1:13" x14ac:dyDescent="0.25">
@@ -19382,12 +19446,12 @@
       <c r="D132" s="110"/>
       <c r="E132" s="110"/>
       <c r="F132" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G132" s="110"/>
       <c r="H132" s="110"/>
       <c r="I132" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J132" s="110">
         <v>6.5</v>
@@ -19397,7 +19461,7 @@
       </c>
       <c r="L132" s="110"/>
       <c r="M132" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="133" spans="1:13" x14ac:dyDescent="0.25">
@@ -19407,12 +19471,12 @@
       <c r="D133" s="110"/>
       <c r="E133" s="110"/>
       <c r="F133" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="G133" s="110"/>
       <c r="H133" s="110"/>
       <c r="I133" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J133" s="110">
         <v>6</v>
@@ -19422,7 +19486,7 @@
       </c>
       <c r="L133" s="110"/>
       <c r="M133" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="134" spans="1:13" x14ac:dyDescent="0.25">
@@ -19432,12 +19496,12 @@
       <c r="D134" s="110"/>
       <c r="E134" s="110"/>
       <c r="F134" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G134" s="110"/>
       <c r="H134" s="110"/>
       <c r="I134" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J134" s="110">
         <v>5.4</v>
@@ -19447,7 +19511,7 @@
       </c>
       <c r="L134" s="110"/>
       <c r="M134" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="135" spans="1:13" x14ac:dyDescent="0.25">
@@ -19457,12 +19521,12 @@
       <c r="D135" s="110"/>
       <c r="E135" s="110"/>
       <c r="F135" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G135" s="110"/>
       <c r="H135" s="110"/>
       <c r="I135" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J135" s="110">
         <v>4.2</v>
@@ -19472,7 +19536,7 @@
       </c>
       <c r="L135" s="110"/>
       <c r="M135" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="136" spans="1:13" x14ac:dyDescent="0.25">
@@ -19499,12 +19563,12 @@
       </c>
       <c r="E137" s="110"/>
       <c r="F137" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="G137" s="110"/>
       <c r="H137" s="110"/>
       <c r="I137" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J137" s="110">
         <v>4</v>
@@ -19514,7 +19578,7 @@
       </c>
       <c r="L137" s="110"/>
       <c r="M137" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="138" spans="1:13" x14ac:dyDescent="0.25">
@@ -19526,12 +19590,12 @@
       </c>
       <c r="E138" s="110"/>
       <c r="F138" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="G138" s="110"/>
       <c r="H138" s="110"/>
       <c r="I138" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J138" s="110">
         <v>4.3</v>
@@ -19541,7 +19605,7 @@
       </c>
       <c r="L138" s="110"/>
       <c r="M138" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="139" spans="1:13" x14ac:dyDescent="0.25">
@@ -19553,12 +19617,12 @@
       </c>
       <c r="E139" s="110"/>
       <c r="F139" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="G139" s="110"/>
       <c r="H139" s="110"/>
       <c r="I139" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J139" s="110">
         <v>4</v>
@@ -19568,7 +19632,7 @@
       </c>
       <c r="L139" s="110"/>
       <c r="M139" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="140" spans="1:13" x14ac:dyDescent="0.25">
@@ -19580,12 +19644,12 @@
       </c>
       <c r="E140" s="110"/>
       <c r="F140" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="G140" s="110"/>
       <c r="H140" s="110"/>
       <c r="I140" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J140" s="110">
         <v>4.3</v>
@@ -19595,7 +19659,7 @@
       </c>
       <c r="L140" s="110"/>
       <c r="M140" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="141" spans="1:13" x14ac:dyDescent="0.25">
@@ -19607,12 +19671,12 @@
       </c>
       <c r="E141" s="110"/>
       <c r="F141" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G141" s="110"/>
       <c r="H141" s="110"/>
       <c r="I141" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J141" s="110">
         <v>4.7</v>
@@ -19622,7 +19686,7 @@
       </c>
       <c r="L141" s="110"/>
       <c r="M141" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="142" spans="1:13" x14ac:dyDescent="0.25">
@@ -19634,12 +19698,12 @@
       </c>
       <c r="E142" s="110"/>
       <c r="F142" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="G142" s="110"/>
       <c r="H142" s="110"/>
       <c r="I142" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J142" s="110">
         <v>3.8</v>
@@ -19649,7 +19713,7 @@
       </c>
       <c r="L142" s="110"/>
       <c r="M142" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="143" spans="1:13" x14ac:dyDescent="0.25">
@@ -19661,12 +19725,12 @@
       </c>
       <c r="E143" s="110"/>
       <c r="F143" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G143" s="110"/>
       <c r="H143" s="110"/>
       <c r="I143" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J143" s="110">
         <v>3.9</v>
@@ -19676,7 +19740,7 @@
       </c>
       <c r="L143" s="110"/>
       <c r="M143" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="144" spans="1:13" x14ac:dyDescent="0.25">
@@ -19688,12 +19752,12 @@
       </c>
       <c r="E144" s="110"/>
       <c r="F144" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G144" s="110"/>
       <c r="H144" s="110"/>
       <c r="I144" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J144" s="110">
         <v>3.2</v>
@@ -19703,7 +19767,7 @@
       </c>
       <c r="L144" s="110"/>
       <c r="M144" s="110" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="145" spans="1:13" x14ac:dyDescent="0.25">
@@ -19730,12 +19794,12 @@
       </c>
       <c r="E146" s="110"/>
       <c r="F146" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="G146" s="110"/>
       <c r="H146" s="110"/>
       <c r="I146" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J146" s="110">
         <v>0</v>
@@ -19744,7 +19808,7 @@
         <v>4</v>
       </c>
       <c r="L146" s="110" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="M146" s="110"/>
     </row>
@@ -19757,12 +19821,12 @@
       </c>
       <c r="E147" s="110"/>
       <c r="F147" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="G147" s="110"/>
       <c r="H147" s="110"/>
       <c r="I147" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J147" s="110">
         <v>0</v>
@@ -19782,12 +19846,12 @@
       </c>
       <c r="E148" s="110"/>
       <c r="F148" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="G148" s="110"/>
       <c r="H148" s="110"/>
       <c r="I148" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J148" s="110">
         <v>0</v>
@@ -19807,12 +19871,12 @@
       </c>
       <c r="E149" s="110"/>
       <c r="F149" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="G149" s="110"/>
       <c r="H149" s="110"/>
       <c r="I149" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J149" s="110">
         <v>0</v>
@@ -19832,12 +19896,12 @@
       </c>
       <c r="E150" s="110"/>
       <c r="F150" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G150" s="110"/>
       <c r="H150" s="110"/>
       <c r="I150" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J150" s="110">
         <v>0</v>
@@ -19857,12 +19921,12 @@
       </c>
       <c r="E151" s="110"/>
       <c r="F151" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="G151" s="110"/>
       <c r="H151" s="110"/>
       <c r="I151" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J151" s="110">
         <v>0</v>
@@ -19882,12 +19946,12 @@
       </c>
       <c r="E152" s="110"/>
       <c r="F152" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G152" s="110"/>
       <c r="H152" s="110"/>
       <c r="I152" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J152" s="110">
         <v>0</v>
@@ -19907,12 +19971,12 @@
       </c>
       <c r="E153" s="110"/>
       <c r="F153" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G153" s="110"/>
       <c r="H153" s="110"/>
       <c r="I153" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J153" s="110">
         <v>0</v>
@@ -19947,12 +20011,12 @@
       </c>
       <c r="E155" s="110"/>
       <c r="F155" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="G155" s="110"/>
       <c r="H155" s="110"/>
       <c r="I155" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J155" s="110">
         <v>0</v>
@@ -19961,7 +20025,7 @@
         <v>4</v>
       </c>
       <c r="L155" s="110" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="M155" s="110"/>
     </row>
@@ -19974,12 +20038,12 @@
       </c>
       <c r="E156" s="110"/>
       <c r="F156" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="G156" s="110"/>
       <c r="H156" s="110"/>
       <c r="I156" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J156" s="110">
         <v>0</v>
@@ -19999,12 +20063,12 @@
       </c>
       <c r="E157" s="110"/>
       <c r="F157" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="G157" s="110"/>
       <c r="H157" s="110"/>
       <c r="I157" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J157" s="110">
         <v>0</v>
@@ -20024,12 +20088,12 @@
       </c>
       <c r="E158" s="110"/>
       <c r="F158" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="G158" s="110"/>
       <c r="H158" s="110"/>
       <c r="I158" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J158" s="110">
         <v>0</v>
@@ -20049,12 +20113,12 @@
       </c>
       <c r="E159" s="110"/>
       <c r="F159" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G159" s="110"/>
       <c r="H159" s="110"/>
       <c r="I159" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J159" s="110">
         <v>0</v>
@@ -20074,12 +20138,12 @@
       </c>
       <c r="E160" s="110"/>
       <c r="F160" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="G160" s="110"/>
       <c r="H160" s="110"/>
       <c r="I160" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J160" s="110">
         <v>0</v>
@@ -20099,12 +20163,12 @@
       </c>
       <c r="E161" s="110"/>
       <c r="F161" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G161" s="110"/>
       <c r="H161" s="110"/>
       <c r="I161" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J161" s="110">
         <v>0</v>
@@ -20124,12 +20188,12 @@
       </c>
       <c r="E162" s="110"/>
       <c r="F162" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G162" s="110"/>
       <c r="H162" s="110"/>
       <c r="I162" s="110" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J162" s="110">
         <v>0</v>
@@ -20165,7 +20229,7 @@
       <c r="G164" s="110"/>
       <c r="H164" s="110"/>
       <c r="I164" s="110" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="J164" s="110">
         <v>0</v>
@@ -20174,7 +20238,7 @@
         <v>9</v>
       </c>
       <c r="L164" s="110" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="M164" s="110"/>
     </row>
@@ -20192,7 +20256,7 @@
       <c r="G165" s="110"/>
       <c r="H165" s="110"/>
       <c r="I165" s="110" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="J165" s="110">
         <v>38</v>
@@ -20202,7 +20266,7 @@
       </c>
       <c r="L165" s="110"/>
       <c r="M165" s="110" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="167" spans="1:13" x14ac:dyDescent="0.25">
@@ -20588,16 +20652,16 @@
         <v>38</v>
       </c>
       <c r="I188" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="J188" s="2">
         <v>78</v>
       </c>
       <c r="K188" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="L188" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="M188" t="s">
         <v>513</v>
@@ -20608,34 +20672,34 @@
         <v>2</v>
       </c>
       <c r="I189" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="J189" s="2">
         <v>81</v>
       </c>
       <c r="K189" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="L189" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="M189" s="258" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="190" spans="1:13" x14ac:dyDescent="0.25">
       <c r="I190" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="J190" s="13">
         <f>18.8*0.13</f>
         <v>2.4440000000000004</v>
       </c>
       <c r="K190" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L190" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="191" spans="1:13" x14ac:dyDescent="0.25">
@@ -20745,7 +20809,7 @@
       </c>
       <c r="J198" s="13">
         <f>INDEX(Foderstater!$X$63:$AI$100,MATCH(E198,Foderstater!$U$63:$U$100,0),MATCH(A198&amp;C198&amp;D198,Foderstater!$X$62:$AI$62,0))</f>
-        <v>38.609681277854051</v>
+        <v>41.480852339300604</v>
       </c>
       <c r="K198" s="159"/>
       <c r="L198" s="159"/>
@@ -20766,7 +20830,7 @@
       </c>
       <c r="J199" s="13">
         <f>INDEX(Foderstater!$X$63:$AI$100,MATCH(E199,Foderstater!$U$63:$U$100,0),MATCH(A199&amp;C199&amp;D199,Foderstater!$X$62:$AI$62,0))</f>
-        <v>9.2377598080515053</v>
+        <v>9.9247167513786927</v>
       </c>
       <c r="K199" s="159"/>
       <c r="L199" s="159"/>
@@ -20850,7 +20914,7 @@
       </c>
       <c r="J203" s="13">
         <f>INDEX(Foderstater!$X$63:$AI$100,MATCH(E203,Foderstater!$U$63:$U$100,0),MATCH(A203&amp;C203&amp;D203,Foderstater!$X$62:$AI$62,0))</f>
-        <v>10.166080013639251</v>
+        <v>6.6079520088655128</v>
       </c>
       <c r="K203" s="159"/>
       <c r="L203" s="159"/>
@@ -21539,7 +21603,7 @@
       </c>
       <c r="J238" s="13">
         <f>INDEX(Foderstater!$X$63:$AI$100,MATCH(E238,Foderstater!$U$63:$U$100,0),MATCH(A238&amp;C238&amp;D238,Foderstater!$X$62:$AI$62,0))</f>
-        <v>20.561419371957058</v>
+        <v>22.93829412577864</v>
       </c>
       <c r="K238" s="159"/>
       <c r="L238" s="159"/>
@@ -21566,7 +21630,7 @@
       </c>
       <c r="J239" s="13">
         <f>INDEX(Foderstater!$X$63:$AI$100,MATCH(E239,Foderstater!$U$63:$U$100,0),MATCH(A239&amp;C239&amp;D239,Foderstater!$X$62:$AI$62,0))</f>
-        <v>9.5364207102254017</v>
+        <v>10.638819198282629</v>
       </c>
       <c r="K239" s="159"/>
       <c r="L239" s="159"/>
@@ -21674,7 +21738,7 @@
       </c>
       <c r="J243" s="13">
         <f>INDEX(Foderstater!$X$63:$AI$100,MATCH(E243,Foderstater!$U$63:$U$100,0),MATCH(A243&amp;C243&amp;D243,Foderstater!$X$62:$AI$62,0))</f>
-        <v>9.9407806910823222</v>
+        <v>6.4615074492035101</v>
       </c>
       <c r="K243" s="159"/>
       <c r="L243" s="159"/>
@@ -23312,7 +23376,7 @@
     </row>
     <row r="318" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A318" s="81" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B318" s="48"/>
       <c r="C318" s="48"/>
@@ -35993,7 +36057,7 @@
       </c>
       <c r="Z2" s="219"/>
       <c r="AA2" s="197" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AB2" s="198"/>
       <c r="AC2" s="198"/>
@@ -36015,7 +36079,7 @@
     </row>
     <row r="3" spans="2:44" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="230" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="C3" s="231"/>
       <c r="D3" s="232" t="s">
@@ -36050,61 +36114,61 @@
       </c>
       <c r="Z3" s="220"/>
       <c r="AA3" s="241" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="AB3" s="202"/>
       <c r="AC3" s="202"/>
-      <c r="AD3" s="265" t="s">
-        <v>525</v>
-      </c>
-      <c r="AE3" s="266" t="s">
-        <v>527</v>
-      </c>
-      <c r="AF3" s="265" t="s">
-        <v>529</v>
-      </c>
-      <c r="AG3" s="266" t="s">
+      <c r="AD3" s="263" t="s">
+        <v>524</v>
+      </c>
+      <c r="AE3" s="264" t="s">
+        <v>526</v>
+      </c>
+      <c r="AF3" s="263" t="s">
+        <v>528</v>
+      </c>
+      <c r="AG3" s="264" t="s">
+        <v>530</v>
+      </c>
+      <c r="AH3" s="263" t="s">
         <v>531</v>
       </c>
-      <c r="AH3" s="265" t="s">
-        <v>532</v>
-      </c>
-      <c r="AI3" s="266" t="s">
+      <c r="AI3" s="264" t="s">
+        <v>533</v>
+      </c>
+      <c r="AJ3" s="263" t="s">
         <v>534</v>
       </c>
-      <c r="AJ3" s="265" t="s">
+      <c r="AK3" s="264" t="s">
         <v>535</v>
       </c>
-      <c r="AK3" s="266" t="s">
-        <v>536</v>
-      </c>
-      <c r="AL3" s="265" t="s">
+      <c r="AL3" s="263" t="s">
+        <v>537</v>
+      </c>
+      <c r="AM3" s="264" t="s">
         <v>538</v>
       </c>
-      <c r="AM3" s="266" t="s">
-        <v>539</v>
-      </c>
-      <c r="AN3" s="265" t="s">
-        <v>559</v>
-      </c>
-      <c r="AO3" s="266" t="s">
+      <c r="AN3" s="263" t="s">
+        <v>558</v>
+      </c>
+      <c r="AO3" s="264" t="s">
+        <v>540</v>
+      </c>
+      <c r="AP3" s="263" t="s">
         <v>541</v>
       </c>
-      <c r="AP3" s="265" t="s">
-        <v>542</v>
-      </c>
-      <c r="AQ3" s="264" t="s">
-        <v>563</v>
-      </c>
-      <c r="AR3" s="263" t="s">
-        <v>558</v>
+      <c r="AQ3" s="262" t="s">
+        <v>562</v>
+      </c>
+      <c r="AR3" s="261" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="4" spans="2:44" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="201"/>
       <c r="C4" s="202"/>
       <c r="D4" s="234" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E4" s="234"/>
       <c r="F4" s="234"/>
@@ -36147,25 +36211,25 @@
       <c r="AA4" s="201"/>
       <c r="AB4" s="202"/>
       <c r="AC4" s="202"/>
-      <c r="AD4" s="265"/>
-      <c r="AE4" s="266"/>
-      <c r="AF4" s="265"/>
-      <c r="AG4" s="266"/>
-      <c r="AH4" s="265"/>
-      <c r="AI4" s="266"/>
-      <c r="AJ4" s="265"/>
-      <c r="AK4" s="266"/>
-      <c r="AL4" s="265"/>
-      <c r="AM4" s="266"/>
-      <c r="AN4" s="265"/>
-      <c r="AO4" s="266"/>
-      <c r="AP4" s="265"/>
-      <c r="AQ4" s="264"/>
-      <c r="AR4" s="263"/>
+      <c r="AD4" s="263"/>
+      <c r="AE4" s="264"/>
+      <c r="AF4" s="263"/>
+      <c r="AG4" s="264"/>
+      <c r="AH4" s="263"/>
+      <c r="AI4" s="264"/>
+      <c r="AJ4" s="263"/>
+      <c r="AK4" s="264"/>
+      <c r="AL4" s="263"/>
+      <c r="AM4" s="264"/>
+      <c r="AN4" s="263"/>
+      <c r="AO4" s="264"/>
+      <c r="AP4" s="263"/>
+      <c r="AQ4" s="262"/>
+      <c r="AR4" s="261"/>
     </row>
     <row r="5" spans="2:44" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="209" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C5" s="210" t="s">
         <v>466</v>
@@ -36242,27 +36306,27 @@
       <c r="AA5" s="201"/>
       <c r="AB5" s="202"/>
       <c r="AC5" s="202"/>
-      <c r="AD5" s="265"/>
-      <c r="AE5" s="266"/>
-      <c r="AF5" s="265"/>
-      <c r="AG5" s="266"/>
-      <c r="AH5" s="265"/>
-      <c r="AI5" s="266"/>
-      <c r="AJ5" s="265"/>
-      <c r="AK5" s="266"/>
-      <c r="AL5" s="265"/>
-      <c r="AM5" s="266"/>
-      <c r="AN5" s="265"/>
-      <c r="AO5" s="266"/>
-      <c r="AP5" s="265"/>
-      <c r="AQ5" s="264"/>
-      <c r="AR5" s="263" t="s">
-        <v>557</v>
+      <c r="AD5" s="263"/>
+      <c r="AE5" s="264"/>
+      <c r="AF5" s="263"/>
+      <c r="AG5" s="264"/>
+      <c r="AH5" s="263"/>
+      <c r="AI5" s="264"/>
+      <c r="AJ5" s="263"/>
+      <c r="AK5" s="264"/>
+      <c r="AL5" s="263"/>
+      <c r="AM5" s="264"/>
+      <c r="AN5" s="263"/>
+      <c r="AO5" s="264"/>
+      <c r="AP5" s="263"/>
+      <c r="AQ5" s="262"/>
+      <c r="AR5" s="261" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="6" spans="2:44" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="201" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C6" s="236">
         <v>1</v>
@@ -36303,7 +36367,7 @@
         <v>1619.5499999999997</v>
       </c>
       <c r="AA6" s="201" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="AB6" s="202"/>
       <c r="AC6" s="202"/>
@@ -36402,55 +36466,55 @@
         <v>751.1500000000002</v>
       </c>
       <c r="AA7" s="201" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="AB7" s="202"/>
       <c r="AC7" s="202"/>
       <c r="AD7" s="207" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="AE7" s="208" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AF7" s="207" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="AG7" s="208" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="AH7" s="207" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="AI7" s="208" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AJ7" s="207" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AK7" s="208" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="AL7" s="207" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="AM7" s="208" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="AN7" s="207" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="AO7" s="208" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="AP7" s="207" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AQ7" s="205"/>
       <c r="AR7" s="206"/>
     </row>
     <row r="8" spans="2:44" x14ac:dyDescent="0.25">
       <c r="B8" s="201" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C8" s="236">
         <v>1</v>
@@ -36540,7 +36604,7 @@
       <c r="Y9" s="225"/>
       <c r="Z9" s="226"/>
       <c r="AA9" s="209" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="AB9" s="202"/>
       <c r="AC9" s="210" t="s">
@@ -36599,7 +36663,7 @@
         <v>1250.5</v>
       </c>
       <c r="AA10" s="201" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="AB10" s="202"/>
       <c r="AC10" s="236">
@@ -36655,7 +36719,7 @@
     </row>
     <row r="11" spans="2:44" x14ac:dyDescent="0.25">
       <c r="B11" s="201" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C11" s="236">
         <v>1</v>
@@ -36692,7 +36756,7 @@
       <c r="Y11" s="225"/>
       <c r="Z11" s="226"/>
       <c r="AA11" s="201" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="AB11" s="202"/>
       <c r="AC11" s="236">
@@ -36722,7 +36786,7 @@
     </row>
     <row r="12" spans="2:44" x14ac:dyDescent="0.25">
       <c r="B12" s="201" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C12" s="236">
         <v>0.85</v>
@@ -36759,7 +36823,7 @@
         <v>244</v>
       </c>
       <c r="AA12" s="201" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="AB12" s="202"/>
       <c r="AC12" s="236">
@@ -36785,7 +36849,7 @@
     </row>
     <row r="13" spans="2:44" x14ac:dyDescent="0.25">
       <c r="B13" s="201" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C13" s="236">
         <v>1</v>
@@ -36844,7 +36908,7 @@
       <c r="Y13" s="225"/>
       <c r="Z13" s="226"/>
       <c r="AA13" s="201" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="AB13" s="202"/>
       <c r="AC13" s="236">
@@ -36870,7 +36934,7 @@
     </row>
     <row r="14" spans="2:44" x14ac:dyDescent="0.25">
       <c r="B14" s="201" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C14" s="236">
         <v>1</v>
@@ -36933,7 +36997,7 @@
         <v>782.99999999999989</v>
       </c>
       <c r="AA14" s="201" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="AB14" s="202"/>
       <c r="AC14" s="236">
@@ -36985,7 +37049,7 @@
     </row>
     <row r="15" spans="2:44" x14ac:dyDescent="0.25">
       <c r="B15" s="201" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="C15" s="236">
         <v>0.86</v>
@@ -37032,7 +37096,7 @@
         <v>1159.4923144269196</v>
       </c>
       <c r="AA15" s="201" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="AB15" s="202"/>
       <c r="AC15" s="236">
@@ -37127,7 +37191,7 @@
       <c r="Y16" s="225"/>
       <c r="Z16" s="226"/>
       <c r="AA16" s="201" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="AB16" s="202"/>
       <c r="AC16" s="236">
@@ -37222,7 +37286,7 @@
         <v>2405.9342126196852</v>
       </c>
       <c r="AA17" s="201" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="AB17" s="202"/>
       <c r="AC17" s="236">
@@ -37387,7 +37451,7 @@
       <c r="Y19" s="225"/>
       <c r="Z19" s="226"/>
       <c r="AA19" s="201" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="AB19" s="202"/>
       <c r="AC19" s="255">
@@ -37516,7 +37580,7 @@
         <v>8279.5672923170714</v>
       </c>
       <c r="AA20" s="201" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="AB20" s="202"/>
       <c r="AC20" s="255">
@@ -37566,7 +37630,7 @@
       <c r="W21" s="42"/>
       <c r="X21" s="42"/>
       <c r="AA21" s="213" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="AB21" s="214"/>
       <c r="AC21" s="214"/>
@@ -37651,7 +37715,7 @@
       <c r="J22" s="165"/>
       <c r="K22" s="165"/>
       <c r="L22" s="174" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M22" s="242"/>
       <c r="N22" s="242"/>
@@ -37691,29 +37755,29 @@
       <c r="N23" s="169"/>
       <c r="O23" s="169"/>
       <c r="P23" s="169"/>
-      <c r="Q23" s="262" t="s">
+      <c r="Q23" s="266" t="s">
+        <v>577</v>
+      </c>
+      <c r="R23" s="266" t="s">
         <v>578</v>
       </c>
-      <c r="R23" s="262" t="s">
-        <v>579</v>
-      </c>
-      <c r="S23" s="262" t="s">
-        <v>566</v>
-      </c>
-      <c r="T23" s="261" t="s">
+      <c r="S23" s="266" t="s">
+        <v>565</v>
+      </c>
+      <c r="T23" s="265" t="s">
         <v>293</v>
       </c>
-      <c r="U23" s="261"/>
-      <c r="V23" s="261" t="s">
+      <c r="U23" s="265"/>
+      <c r="V23" s="265" t="s">
         <v>294</v>
       </c>
-      <c r="W23" s="261"/>
+      <c r="W23" s="265"/>
       <c r="X23" s="168" t="s">
         <v>465</v>
       </c>
       <c r="Y23" s="165"/>
       <c r="Z23" s="174" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AA23" s="83"/>
       <c r="AB23" s="83"/>
@@ -37732,9 +37796,9 @@
       <c r="P24" s="170" t="s">
         <v>466</v>
       </c>
-      <c r="Q24" s="262"/>
-      <c r="R24" s="262"/>
-      <c r="S24" s="262"/>
+      <c r="Q24" s="266"/>
+      <c r="R24" s="266"/>
+      <c r="S24" s="266"/>
       <c r="T24" s="244" t="s">
         <v>466</v>
       </c>
@@ -37751,7 +37815,7 @@
         <v>500</v>
       </c>
       <c r="Z24" s="174" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA24" s="169"/>
       <c r="AB24" s="169"/>
@@ -37856,7 +37920,7 @@
     </row>
     <row r="26" spans="2:44" x14ac:dyDescent="0.25">
       <c r="B26" s="174" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="C26" s="174"/>
       <c r="D26" s="168"/>
@@ -38644,7 +38708,7 @@
         <v>0</v>
       </c>
       <c r="L34" s="169" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="M34" s="169"/>
       <c r="N34" s="169"/>
@@ -38940,7 +39004,7 @@
         <v>1</v>
       </c>
       <c r="L38" s="169" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="M38" s="169"/>
       <c r="N38" s="169"/>
@@ -39404,7 +39468,7 @@
         <v>0.40587012896078656</v>
       </c>
       <c r="L44" s="169" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="M44" s="169"/>
       <c r="N44" s="169"/>
@@ -39481,7 +39545,7 @@
         <v>0.2671631311304497</v>
       </c>
       <c r="L45" s="169" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="M45" s="169"/>
       <c r="N45" s="169"/>
@@ -39558,7 +39622,7 @@
         <v>0.14385536511797675</v>
       </c>
       <c r="L46" s="169" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="M46" s="169"/>
       <c r="N46" s="169"/>
@@ -39636,7 +39700,7 @@
         <v>0.46986991038291381</v>
       </c>
       <c r="L47" s="169" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="M47" s="169"/>
       <c r="N47" s="169"/>
@@ -39779,7 +39843,7 @@
         <v>0.15455308043620117</v>
       </c>
       <c r="L49" s="169" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="M49" s="169"/>
       <c r="N49" s="169"/>
@@ -39820,7 +39884,7 @@
     </row>
     <row r="50" spans="2:44" x14ac:dyDescent="0.25">
       <c r="L50" s="169" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="M50" s="169"/>
       <c r="N50" s="169"/>
@@ -39945,7 +40009,7 @@
     </row>
     <row r="53" spans="2:44" x14ac:dyDescent="0.25">
       <c r="L53" s="169" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="M53" s="169"/>
       <c r="N53" s="169"/>
@@ -40024,10 +40088,14 @@
         <f t="shared" si="11"/>
         <v>0.93</v>
       </c>
+      <c r="Z54" s="271"/>
+      <c r="AA54" s="272"/>
+      <c r="AB54" s="273"/>
+      <c r="AC54" s="274"/>
     </row>
     <row r="55" spans="2:44" x14ac:dyDescent="0.25">
       <c r="L55" s="169" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="M55" s="169"/>
       <c r="N55" s="169"/>
@@ -40100,16 +40168,40 @@
         <f t="shared" si="11"/>
         <v>0.93</v>
       </c>
+      <c r="Z56" s="268" t="s">
+        <v>621</v>
+      </c>
+      <c r="AA56" s="268"/>
+      <c r="AB56" s="268"/>
+      <c r="AC56" s="267"/>
+      <c r="AE56" t="s">
+        <v>622</v>
+      </c>
       <c r="AQ56" s="12"/>
       <c r="AR56" s="26"/>
     </row>
     <row r="57" spans="2:44" x14ac:dyDescent="0.25">
+      <c r="Z57" s="268" t="s">
+        <v>623</v>
+      </c>
+      <c r="AA57" s="268"/>
+      <c r="AB57" s="268"/>
+      <c r="AC57" s="267"/>
+      <c r="AE57" t="s">
+        <v>1</v>
+      </c>
+      <c r="AG57">
+        <v>9</v>
+      </c>
+      <c r="AH57" t="s">
+        <v>9</v>
+      </c>
       <c r="AQ57" s="12"/>
       <c r="AR57" s="26"/>
     </row>
     <row r="58" spans="2:44" x14ac:dyDescent="0.25">
       <c r="S58" s="185" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="T58" s="12">
         <f>SUM(T25:T30)</f>
@@ -40127,12 +40219,28 @@
         <f>V58/SUM(V$58:V$59)</f>
         <v>0.68124800328654078</v>
       </c>
+      <c r="Z58" s="267" t="s">
+        <v>617</v>
+      </c>
+      <c r="AA58" s="268"/>
+      <c r="AB58" s="268"/>
+      <c r="AC58" s="267"/>
+      <c r="AE58" t="s">
+        <v>5</v>
+      </c>
+      <c r="AG58">
+        <v>14</v>
+      </c>
+      <c r="AH58" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI58" s="2"/>
       <c r="AQ58" s="12"/>
       <c r="AR58" s="26"/>
     </row>
     <row r="59" spans="2:44" x14ac:dyDescent="0.25">
       <c r="S59" s="185" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="T59" s="12">
         <f>SUM(T31:T55)</f>
@@ -40153,8 +40261,100 @@
       <c r="AQ59" s="12"/>
       <c r="AR59" s="26"/>
     </row>
+    <row r="60" spans="2:44" x14ac:dyDescent="0.25">
+      <c r="W60" s="269" t="s">
+        <v>618</v>
+      </c>
+      <c r="X60" s="270">
+        <v>1</v>
+      </c>
+      <c r="Y60" s="270">
+        <v>1</v>
+      </c>
+      <c r="Z60" s="270">
+        <v>1</v>
+      </c>
+      <c r="AA60" s="270">
+        <v>1</v>
+      </c>
+      <c r="AB60" s="270">
+        <v>1</v>
+      </c>
+      <c r="AC60" s="270">
+        <v>1</v>
+      </c>
+      <c r="AD60" s="270">
+        <v>0.65</v>
+      </c>
+      <c r="AE60" s="270">
+        <v>1</v>
+      </c>
+      <c r="AF60" s="270">
+        <v>1</v>
+      </c>
+      <c r="AG60" s="270">
+        <v>1</v>
+      </c>
+      <c r="AH60" s="270">
+        <v>0.65</v>
+      </c>
+      <c r="AI60" s="270">
+        <v>1</v>
+      </c>
+    </row>
     <row r="61" spans="2:44" x14ac:dyDescent="0.25">
       <c r="T61" s="2"/>
+      <c r="W61" s="269" t="s">
+        <v>619</v>
+      </c>
+      <c r="X61" s="270">
+        <f>1+(D71*(1-X60))/SUM(D66:D67)</f>
+        <v>1</v>
+      </c>
+      <c r="Y61" s="270">
+        <f t="shared" ref="X61:AI61" si="14">1+(E71*(1-Y60))/SUM(E66:E67)</f>
+        <v>1</v>
+      </c>
+      <c r="Z61" s="270">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AA61" s="270">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AB61" s="270">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AC61" s="270">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AD61" s="270">
+        <f t="shared" si="14"/>
+        <v>1.0743640187232888</v>
+      </c>
+      <c r="AE61" s="270">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AF61" s="270">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AG61" s="270">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AH61" s="270">
+        <f t="shared" si="14"/>
+        <v>1.1155987682962838</v>
+      </c>
+      <c r="AI61" s="270">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="62" spans="2:44" x14ac:dyDescent="0.25">
       <c r="B62" s="6" t="s">
@@ -40261,25 +40461,26 @@
       <c r="O63" t="s">
         <v>416</v>
       </c>
+      <c r="Q63" s="4"/>
       <c r="T63" s="2"/>
       <c r="U63" s="110" t="str">
         <f>B66</f>
         <v>ley silage, 1st cut</v>
       </c>
       <c r="X63" s="13">
-        <f t="shared" ref="X63:X68" si="14">D66/D$116*100</f>
+        <f>X61*D66/D$116*100</f>
         <v>0</v>
       </c>
       <c r="Y63" s="13">
-        <f t="shared" ref="Y63:AI63" si="15">E66/E$116*100</f>
+        <f>Y61*E66/E$116*100</f>
         <v>55.38698659192309</v>
       </c>
       <c r="Z63" s="13">
-        <f t="shared" si="15"/>
+        <f>Z61*F66/F$116*100</f>
         <v>0</v>
       </c>
       <c r="AA63" s="13">
-        <f t="shared" si="15"/>
+        <f t="shared" ref="Y63:AI63" si="15">AA61*G66/G$116*100</f>
         <v>0</v>
       </c>
       <c r="AB63" s="13">
@@ -40292,7 +40493,7 @@
       </c>
       <c r="AD63" s="13">
         <f t="shared" si="15"/>
-        <v>38.609681277854051</v>
+        <v>41.480852339300604</v>
       </c>
       <c r="AE63" s="13">
         <f t="shared" si="15"/>
@@ -40308,7 +40509,7 @@
       </c>
       <c r="AH63" s="13">
         <f t="shared" si="15"/>
-        <v>20.561419371957058</v>
+        <v>22.93829412577864</v>
       </c>
       <c r="AI63" s="13">
         <f t="shared" si="15"/>
@@ -40362,51 +40563,51 @@
         <v>ley silage, regrowth</v>
       </c>
       <c r="X64" s="13">
-        <f t="shared" si="14"/>
+        <f>X61*D67/D$116*100</f>
         <v>19.638470390756044</v>
       </c>
       <c r="Y64" s="13">
-        <f t="shared" ref="Y64:AI64" si="17">E67/E$116*100</f>
+        <f>Y61*E67/E$116*100</f>
         <v>0</v>
       </c>
       <c r="Z64" s="13">
-        <f t="shared" si="17"/>
+        <f>Z61*F67/F$116*100</f>
         <v>68.854768967576106</v>
       </c>
       <c r="AA64" s="13">
-        <f t="shared" si="17"/>
+        <f>AA61*G67/G$116*100</f>
         <v>69.016974351370379</v>
       </c>
       <c r="AB64" s="13">
-        <f t="shared" si="17"/>
+        <f>AB61*H67/H$116*100</f>
         <v>0</v>
       </c>
       <c r="AC64" s="13">
-        <f t="shared" si="17"/>
+        <f>AC61*I67/I$116*100</f>
         <v>0</v>
       </c>
       <c r="AD64" s="13">
-        <f t="shared" si="17"/>
-        <v>9.2377598080515053</v>
+        <f>AD61*J67/J$116*100</f>
+        <v>9.9247167513786927</v>
       </c>
       <c r="AE64" s="13">
-        <f t="shared" si="17"/>
+        <f>AE61*K67/K$116*100</f>
         <v>0</v>
       </c>
       <c r="AF64" s="13">
-        <f t="shared" si="17"/>
+        <f>AF61*L67/L$116*100</f>
         <v>55.029062371648976</v>
       </c>
       <c r="AG64" s="13">
-        <f t="shared" si="17"/>
+        <f>AG61*M67/M$116*100</f>
         <v>0</v>
       </c>
       <c r="AH64" s="13">
-        <f t="shared" si="17"/>
-        <v>9.5364207102254017</v>
+        <f>AH61*N67/N$116*100</f>
+        <v>10.638819198282629</v>
       </c>
       <c r="AI64" s="13">
-        <f t="shared" si="17"/>
+        <f>AI61*O67/O$116*100</f>
         <v>0</v>
       </c>
     </row>
@@ -40421,7 +40622,7 @@
         <v>other silage</v>
       </c>
       <c r="X65" s="13">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="X63:X68" si="17">D68/D$116*100</f>
         <v>20.321711421281208</v>
       </c>
       <c r="Y65" s="13">
@@ -40510,14 +40711,13 @@
         <f>N9*C9</f>
         <v>1868</v>
       </c>
-      <c r="Q66" s="2"/>
       <c r="T66" s="72"/>
       <c r="U66" s="110" t="str">
         <f t="shared" si="16"/>
         <v>maize silage</v>
       </c>
       <c r="X66" s="13">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="Y66" s="13">
@@ -40596,14 +40796,12 @@
         <f>Z7</f>
         <v>751.1500000000002</v>
       </c>
-      <c r="Q67" s="2"/>
-      <c r="T67" s="2"/>
       <c r="U67" s="110" t="str">
         <f t="shared" si="16"/>
         <v>straw</v>
       </c>
       <c r="X67" s="13">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>1.1297448457337229</v>
       </c>
       <c r="Y67" s="13">
@@ -40666,18 +40864,16 @@
       <c r="L68" s="12"/>
       <c r="M68" s="12"/>
       <c r="N68" s="12"/>
-      <c r="Q68" s="2"/>
-      <c r="T68" s="2"/>
       <c r="U68" s="110" t="str">
         <f t="shared" si="16"/>
         <v>grazing</v>
       </c>
       <c r="X68" s="13">
-        <f t="shared" si="14"/>
+        <f>X60*D71/D$116*100</f>
         <v>58.050981669759572</v>
       </c>
       <c r="Y68" s="13">
-        <f t="shared" ref="Y68:AI68" si="21">E71/E$116*100</f>
+        <f t="shared" ref="Y68:AI68" si="21">Y60*E71/E$116*100</f>
         <v>21.161076246926353</v>
       </c>
       <c r="Z68" s="13">
@@ -40698,7 +40894,7 @@
       </c>
       <c r="AD68" s="13">
         <f t="shared" si="21"/>
-        <v>10.166080013639251</v>
+        <v>6.6079520088655128</v>
       </c>
       <c r="AE68" s="13">
         <f t="shared" si="21"/>
@@ -40714,7 +40910,7 @@
       </c>
       <c r="AH68" s="13">
         <f t="shared" si="21"/>
-        <v>9.9407806910823222</v>
+        <v>6.4615074492035101</v>
       </c>
       <c r="AI68" s="13">
         <f t="shared" si="21"/>
@@ -40743,8 +40939,6 @@
         <f>N10*C10</f>
         <v>436</v>
       </c>
-      <c r="Q69" s="2"/>
-      <c r="T69" s="2"/>
       <c r="U69" s="110" t="str">
         <f t="shared" ref="U69:U100" si="22">B82</f>
         <v>wheat</v>
@@ -40819,8 +41013,6 @@
         <f>Z12</f>
         <v>244</v>
       </c>
-      <c r="Q70" s="2"/>
-      <c r="T70" s="2"/>
       <c r="U70" s="110" t="str">
         <f t="shared" si="22"/>
         <v>barley</v>
@@ -43833,7 +44025,7 @@
         <v>rye bran</v>
       </c>
       <c r="E104" s="13">
-        <f t="shared" si="46"/>
+        <f>E$81*$W47</f>
         <v>8.8218496845068217E-2</v>
       </c>
       <c r="H104" s="13">
@@ -43869,14 +44061,14 @@
       <c r="U104" s="6"/>
       <c r="V104" s="6"/>
       <c r="W104" s="185" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="X104" s="72">
-        <f t="shared" ref="X104:AI104" si="94">SUM(X63:X68)</f>
+        <f>SUM(X63:X68)</f>
         <v>99.140908327530553</v>
       </c>
       <c r="Y104" s="72">
-        <f t="shared" si="94"/>
+        <f t="shared" ref="X104:AI104" si="94">SUM(Y63:Y68)</f>
         <v>76.548062838849447</v>
       </c>
       <c r="Z104" s="72">
@@ -43897,7 +44089,7 @@
       </c>
       <c r="AD104" s="72">
         <f t="shared" si="94"/>
-        <v>61.18149494798412</v>
+        <v>61.181494947984113</v>
       </c>
       <c r="AE104" s="72">
         <f t="shared" si="94"/>
@@ -43959,6 +44151,57 @@
         <v>5.677922096367217</v>
       </c>
       <c r="Q105" s="2"/>
+      <c r="W105" s="185" t="s">
+        <v>620</v>
+      </c>
+      <c r="X105" s="72">
+        <f>X68/X104*100</f>
+        <v>58.5540143307718</v>
+      </c>
+      <c r="Y105" s="72">
+        <f t="shared" ref="Y105:AI105" si="97">Y68/Y104*100</f>
+        <v>27.644169508868021</v>
+      </c>
+      <c r="Z105" s="72">
+        <f t="shared" si="97"/>
+        <v>30.646316743875307</v>
+      </c>
+      <c r="AA105" s="72">
+        <f t="shared" si="97"/>
+        <v>30.495841704076714</v>
+      </c>
+      <c r="AB105" s="72">
+        <f t="shared" si="97"/>
+        <v>0</v>
+      </c>
+      <c r="AC105" s="72">
+        <f t="shared" si="97"/>
+        <v>0</v>
+      </c>
+      <c r="AD105" s="72">
+        <f t="shared" si="97"/>
+        <v>10.800572974693617</v>
+      </c>
+      <c r="AE105" s="72">
+        <f t="shared" si="97"/>
+        <v>16.294245990112653</v>
+      </c>
+      <c r="AF105" s="72">
+        <f t="shared" si="97"/>
+        <v>41.235797089451033</v>
+      </c>
+      <c r="AG105" s="72">
+        <f t="shared" si="97"/>
+        <v>0</v>
+      </c>
+      <c r="AH105" s="72">
+        <f t="shared" si="97"/>
+        <v>10.949399767651991</v>
+      </c>
+      <c r="AI105" s="72">
+        <f t="shared" si="97"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="106" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B106" t="str">
@@ -43979,23 +44222,23 @@
         <v>0</v>
       </c>
       <c r="K106" s="13">
-        <f t="shared" ref="K106:M106" si="97">K$81*$W49</f>
+        <f t="shared" ref="K106:M106" si="98">K$81*$W49</f>
         <v>0</v>
       </c>
       <c r="L106" s="13">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>0</v>
       </c>
       <c r="M106" s="13">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>0</v>
       </c>
       <c r="N106" s="13">
-        <f t="shared" ref="N106:O106" si="98">N$81*$U49</f>
+        <f t="shared" ref="N106:O106" si="99">N$81*$U49</f>
         <v>0</v>
       </c>
       <c r="O106" s="13">
-        <f t="shared" si="98"/>
+        <f t="shared" si="99"/>
         <v>0</v>
       </c>
       <c r="Q106" s="2"/>
@@ -44019,23 +44262,23 @@
         <v>3.3062241528984204</v>
       </c>
       <c r="K107" s="13">
-        <f t="shared" ref="K107:M107" si="99">K$81*$W50</f>
+        <f t="shared" ref="K107:M107" si="100">K$81*$W50</f>
         <v>5.3579732624603534E-2</v>
       </c>
       <c r="L107" s="13">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>0.12681195334591416</v>
       </c>
       <c r="M107" s="13">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>0.25884226195508947</v>
       </c>
       <c r="N107" s="13">
-        <f t="shared" ref="N107:O107" si="100">N$81*$U50</f>
+        <f t="shared" ref="N107:O107" si="101">N$81*$U50</f>
         <v>5.2251098750790144</v>
       </c>
       <c r="O107" s="13">
-        <f t="shared" si="100"/>
+        <f t="shared" si="101"/>
         <v>0.17156898055071318</v>
       </c>
       <c r="Q107" s="2"/>
@@ -44059,23 +44302,23 @@
         <v>36.664020794401559</v>
       </c>
       <c r="K108" s="13">
-        <f t="shared" ref="K108:M108" si="101">K$81*$W51</f>
+        <f t="shared" ref="K108:M108" si="102">K$81*$W51</f>
         <v>0.59416674135200243</v>
       </c>
       <c r="L108" s="13">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>1.4062676574355435</v>
       </c>
       <c r="M108" s="13">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>2.8704037100665714</v>
       </c>
       <c r="N108" s="13">
-        <f t="shared" ref="N108:O108" si="102">N$81*$U51</f>
+        <f t="shared" ref="N108:O108" si="103">N$81*$U51</f>
         <v>57.943299744206961</v>
       </c>
       <c r="O108" s="13">
-        <f t="shared" si="102"/>
+        <f t="shared" si="103"/>
         <v>1.9025959462158974</v>
       </c>
       <c r="Q108" s="2"/>
@@ -44099,23 +44342,23 @@
         <v>70.746128085415293</v>
       </c>
       <c r="K109" s="13">
-        <f t="shared" ref="K109:M109" si="103">K$81*$W52</f>
+        <f t="shared" ref="K109:M109" si="104">K$81*$W52</f>
         <v>1.1464917234118837</v>
       </c>
       <c r="L109" s="13">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>2.7135046746019542</v>
       </c>
       <c r="M109" s="13">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>5.5386709948688679</v>
       </c>
       <c r="N109" s="13">
-        <f t="shared" ref="N109:O109" si="104">N$81*$U52</f>
+        <f t="shared" ref="N109:O109" si="105">N$81*$U52</f>
         <v>111.80617991633959</v>
       </c>
       <c r="O109" s="13">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>3.6712093651860145</v>
       </c>
       <c r="Q109" s="2"/>
@@ -44139,23 +44382,23 @@
         <v>0</v>
       </c>
       <c r="K110" s="13">
-        <f t="shared" ref="K110:M110" si="105">K$81*$W53</f>
+        <f t="shared" ref="K110:M110" si="106">K$81*$W53</f>
         <v>0</v>
       </c>
       <c r="L110" s="13">
-        <f t="shared" si="105"/>
+        <f t="shared" si="106"/>
         <v>0</v>
       </c>
       <c r="M110" s="13">
-        <f t="shared" si="105"/>
+        <f t="shared" si="106"/>
         <v>0</v>
       </c>
       <c r="N110" s="13">
-        <f t="shared" ref="N110:O110" si="106">N$81*$U53</f>
+        <f t="shared" ref="N110:O110" si="107">N$81*$U53</f>
         <v>0</v>
       </c>
       <c r="O110" s="13">
-        <f t="shared" si="106"/>
+        <f t="shared" si="107"/>
         <v>0</v>
       </c>
       <c r="Q110" s="2"/>
@@ -44179,23 +44422,23 @@
         <v>0.32389393208400408</v>
       </c>
       <c r="K111" s="13">
-        <f t="shared" ref="K111:M111" si="107">K$81*$W54</f>
+        <f t="shared" ref="K111:M111" si="108">K$81*$W54</f>
         <v>5.2489333684707425E-3</v>
       </c>
       <c r="L111" s="13">
-        <f t="shared" si="107"/>
+        <f t="shared" si="108"/>
         <v>1.2423120848734343E-2</v>
       </c>
       <c r="M111" s="13">
-        <f t="shared" si="107"/>
+        <f t="shared" si="108"/>
         <v>2.5357457370413061E-2</v>
       </c>
       <c r="N111" s="13">
-        <f t="shared" ref="N111:O111" si="108">N$81*$U54</f>
+        <f t="shared" ref="N111:O111" si="109">N$81*$U54</f>
         <v>0.51187738784336978</v>
       </c>
       <c r="O111" s="13">
-        <f t="shared" si="108"/>
+        <f t="shared" si="109"/>
         <v>1.6807738726818816E-2</v>
       </c>
       <c r="Q111" s="2"/>
@@ -44219,23 +44462,23 @@
         <v>0</v>
       </c>
       <c r="K112" s="13">
-        <f t="shared" ref="K112:M112" si="109">K$81*$W55</f>
+        <f t="shared" ref="K112:M112" si="110">K$81*$W55</f>
         <v>0</v>
       </c>
       <c r="L112" s="13">
-        <f t="shared" si="109"/>
+        <f t="shared" si="110"/>
         <v>0</v>
       </c>
       <c r="M112" s="13">
-        <f t="shared" si="109"/>
+        <f t="shared" si="110"/>
         <v>0</v>
       </c>
       <c r="N112" s="13">
-        <f t="shared" ref="N112:O112" si="110">N$81*$U55</f>
+        <f t="shared" ref="N112:O112" si="111">N$81*$U55</f>
         <v>0</v>
       </c>
       <c r="O112" s="13">
-        <f t="shared" si="110"/>
+        <f t="shared" si="111"/>
         <v>0</v>
       </c>
       <c r="Q112" s="2"/>
@@ -44314,11 +44557,11 @@
         <v>3614.2395719012102</v>
       </c>
       <c r="G116" s="12">
-        <f t="shared" ref="G116:O116" si="111">SUM(G66:G71,G73:G77,G79:G80,G82:G113)</f>
+        <f t="shared" ref="G116:O116" si="112">SUM(G66:G71,G73:G77,G79:G80,G82:G113)</f>
         <v>3674.463258325256</v>
       </c>
       <c r="H116" s="12">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>2068.2399000680466</v>
       </c>
       <c r="I116" s="12">
@@ -44326,32 +44569,37 @@
         <v>2077.7399999999998</v>
       </c>
       <c r="J116" s="12">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>7702.0837820427678</v>
       </c>
       <c r="K116" s="12">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>1359.3600606369851</v>
       </c>
       <c r="L116" s="12">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>4800.5181359476801</v>
       </c>
       <c r="M116" s="12">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>3259.6633994882459</v>
       </c>
       <c r="N116" s="12">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>7876.6449470353336</v>
       </c>
       <c r="O116" s="12">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>3296.3399999999992</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="V23:W23"/>
+    <mergeCell ref="T23:U23"/>
+    <mergeCell ref="Q23:Q24"/>
+    <mergeCell ref="R23:R24"/>
+    <mergeCell ref="S23:S24"/>
     <mergeCell ref="AR3:AR5"/>
     <mergeCell ref="AQ3:AQ5"/>
     <mergeCell ref="AD3:AD5"/>
@@ -44367,17 +44615,12 @@
     <mergeCell ref="AN3:AN5"/>
     <mergeCell ref="AO3:AO5"/>
     <mergeCell ref="AP3:AP5"/>
-    <mergeCell ref="V23:W23"/>
-    <mergeCell ref="T23:U23"/>
-    <mergeCell ref="Q23:Q24"/>
-    <mergeCell ref="R23:R24"/>
-    <mergeCell ref="S23:S24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="S39:S56 F67:G67 L71 E81 S25:S38" formulaRange="1"/>
-    <ignoredError sqref="V39:V56 AF62 J73:J76 N73:N76 V25:V38 F28" formula="1"/>
+    <ignoredError sqref="V39:V56 J73:J76 N73:N76 V25:V38 F28" formula="1"/>
   </ignoredErrors>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>

</xml_diff>

<commit_message>
Small adjustments in data incl tomato & cucumber imports
</commit_message>
<xml_diff>
--- a/data/default/CattleHerd.xlsx
+++ b/data/default/CattleHerd.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18360" windowHeight="6705" tabRatio="846" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18360" windowHeight="6705" tabRatio="846" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="13" r:id="rId1"/>
@@ -2046,7 +2046,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="48" x14ac:knownFonts="1">
+  <fonts count="49" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2395,6 +2395,13 @@
     <font>
       <sz val="11"/>
       <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3009,7 +3016,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="279">
+  <cellXfs count="281">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3457,6 +3464,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -40654,54 +40665,54 @@
     </row>
     <row r="61" spans="2:44" x14ac:dyDescent="0.25">
       <c r="T61" s="2"/>
-      <c r="W61" s="263" t="s">
+      <c r="W61" s="279" t="s">
         <v>618</v>
       </c>
-      <c r="X61" s="264">
+      <c r="X61" s="280">
         <f>1+(D71*(1-X60))/SUM(D66:D67)</f>
         <v>1</v>
       </c>
-      <c r="Y61" s="264">
+      <c r="Y61" s="280">
         <f t="shared" ref="Y61:AI61" si="14">1+(E71*(1-Y60))/SUM(E66:E67)</f>
         <v>1</v>
       </c>
-      <c r="Z61" s="264">
+      <c r="Z61" s="280">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>
-      <c r="AA61" s="264">
+      <c r="AA61" s="280">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>
-      <c r="AB61" s="264">
+      <c r="AB61" s="280">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>
-      <c r="AC61" s="264">
+      <c r="AC61" s="280">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>
-      <c r="AD61" s="264">
+      <c r="AD61" s="280">
         <f t="shared" si="14"/>
         <v>1.0743640187232888</v>
       </c>
-      <c r="AE61" s="264">
+      <c r="AE61" s="280">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>
-      <c r="AF61" s="264">
+      <c r="AF61" s="280">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>
-      <c r="AG61" s="264">
+      <c r="AG61" s="280">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>
-      <c r="AH61" s="264">
+      <c r="AH61" s="280">
         <f t="shared" si="14"/>
         <v>1.1155987682962838</v>
       </c>
-      <c r="AI61" s="264">
+      <c r="AI61" s="280">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
First step adjusting feed req. calc (need to check)
</commit_message>
<xml_diff>
--- a/data/default/CattleHerd.xlsx
+++ b/data/default/CattleHerd.xlsx
@@ -56,7 +56,7 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId12"/>
+    <pivotCache cacheId="1" r:id="rId12"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -144,7 +144,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4270" uniqueCount="635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4273" uniqueCount="635">
   <si>
     <t>value</t>
   </si>
@@ -3034,7 +3034,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="282">
+  <cellXfs count="290">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3468,6 +3468,19 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3486,7 +3499,6 @@
     <xf numFmtId="0" fontId="40" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -15103,7 +15115,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="L3:O43" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="12">
     <pivotField axis="axisRow" showAll="0">
@@ -17812,7 +17824,7 @@
       <c r="I51" s="110" t="s">
         <v>633</v>
       </c>
-      <c r="J51" s="281">
+      <c r="J51" s="275">
         <v>100</v>
       </c>
       <c r="K51" t="s">
@@ -18061,7 +18073,7 @@
       <c r="I61" s="110" t="s">
         <v>633</v>
       </c>
-      <c r="J61" s="281">
+      <c r="J61" s="275">
         <v>300</v>
       </c>
       <c r="K61" t="s">
@@ -18084,7 +18096,7 @@
       <c r="I62" s="110" t="s">
         <v>634</v>
       </c>
-      <c r="J62" s="281">
+      <c r="J62" s="275">
         <v>275</v>
       </c>
       <c r="K62" t="s">
@@ -36525,49 +36537,49 @@
       </c>
       <c r="AB3" s="202"/>
       <c r="AC3" s="202"/>
-      <c r="AD3" s="279" t="s">
+      <c r="AD3" s="288" t="s">
         <v>520</v>
       </c>
-      <c r="AE3" s="280" t="s">
+      <c r="AE3" s="289" t="s">
         <v>522</v>
       </c>
-      <c r="AF3" s="279" t="s">
+      <c r="AF3" s="288" t="s">
         <v>524</v>
       </c>
-      <c r="AG3" s="280" t="s">
+      <c r="AG3" s="289" t="s">
         <v>526</v>
       </c>
-      <c r="AH3" s="279" t="s">
+      <c r="AH3" s="288" t="s">
         <v>527</v>
       </c>
-      <c r="AI3" s="280" t="s">
+      <c r="AI3" s="289" t="s">
         <v>529</v>
       </c>
-      <c r="AJ3" s="279" t="s">
+      <c r="AJ3" s="288" t="s">
         <v>530</v>
       </c>
-      <c r="AK3" s="280" t="s">
+      <c r="AK3" s="289" t="s">
         <v>531</v>
       </c>
-      <c r="AL3" s="279" t="s">
+      <c r="AL3" s="288" t="s">
         <v>533</v>
       </c>
-      <c r="AM3" s="280" t="s">
+      <c r="AM3" s="289" t="s">
         <v>534</v>
       </c>
-      <c r="AN3" s="279" t="s">
+      <c r="AN3" s="288" t="s">
         <v>554</v>
       </c>
-      <c r="AO3" s="280" t="s">
+      <c r="AO3" s="289" t="s">
         <v>536</v>
       </c>
-      <c r="AP3" s="279" t="s">
+      <c r="AP3" s="288" t="s">
         <v>537</v>
       </c>
-      <c r="AQ3" s="278" t="s">
+      <c r="AQ3" s="287" t="s">
         <v>558</v>
       </c>
-      <c r="AR3" s="277" t="s">
+      <c r="AR3" s="286" t="s">
         <v>553</v>
       </c>
     </row>
@@ -36618,21 +36630,21 @@
       <c r="AA4" s="201"/>
       <c r="AB4" s="202"/>
       <c r="AC4" s="202"/>
-      <c r="AD4" s="279"/>
-      <c r="AE4" s="280"/>
-      <c r="AF4" s="279"/>
-      <c r="AG4" s="280"/>
-      <c r="AH4" s="279"/>
-      <c r="AI4" s="280"/>
-      <c r="AJ4" s="279"/>
-      <c r="AK4" s="280"/>
-      <c r="AL4" s="279"/>
-      <c r="AM4" s="280"/>
-      <c r="AN4" s="279"/>
-      <c r="AO4" s="280"/>
-      <c r="AP4" s="279"/>
-      <c r="AQ4" s="278"/>
-      <c r="AR4" s="277"/>
+      <c r="AD4" s="288"/>
+      <c r="AE4" s="289"/>
+      <c r="AF4" s="288"/>
+      <c r="AG4" s="289"/>
+      <c r="AH4" s="288"/>
+      <c r="AI4" s="289"/>
+      <c r="AJ4" s="288"/>
+      <c r="AK4" s="289"/>
+      <c r="AL4" s="288"/>
+      <c r="AM4" s="289"/>
+      <c r="AN4" s="288"/>
+      <c r="AO4" s="289"/>
+      <c r="AP4" s="288"/>
+      <c r="AQ4" s="287"/>
+      <c r="AR4" s="286"/>
     </row>
     <row r="5" spans="2:44" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="209" t="s">
@@ -36713,21 +36725,21 @@
       <c r="AA5" s="201"/>
       <c r="AB5" s="202"/>
       <c r="AC5" s="202"/>
-      <c r="AD5" s="279"/>
-      <c r="AE5" s="280"/>
-      <c r="AF5" s="279"/>
-      <c r="AG5" s="280"/>
-      <c r="AH5" s="279"/>
-      <c r="AI5" s="280"/>
-      <c r="AJ5" s="279"/>
-      <c r="AK5" s="280"/>
-      <c r="AL5" s="279"/>
-      <c r="AM5" s="280"/>
-      <c r="AN5" s="279"/>
-      <c r="AO5" s="280"/>
-      <c r="AP5" s="279"/>
-      <c r="AQ5" s="278"/>
-      <c r="AR5" s="277" t="s">
+      <c r="AD5" s="288"/>
+      <c r="AE5" s="289"/>
+      <c r="AF5" s="288"/>
+      <c r="AG5" s="289"/>
+      <c r="AH5" s="288"/>
+      <c r="AI5" s="289"/>
+      <c r="AJ5" s="288"/>
+      <c r="AK5" s="289"/>
+      <c r="AL5" s="288"/>
+      <c r="AM5" s="289"/>
+      <c r="AN5" s="288"/>
+      <c r="AO5" s="289"/>
+      <c r="AP5" s="288"/>
+      <c r="AQ5" s="287"/>
+      <c r="AR5" s="286" t="s">
         <v>552</v>
       </c>
     </row>
@@ -38162,23 +38174,23 @@
       <c r="N23" s="169"/>
       <c r="O23" s="169"/>
       <c r="P23" s="169"/>
-      <c r="Q23" s="276" t="s">
+      <c r="Q23" s="285" t="s">
         <v>573</v>
       </c>
-      <c r="R23" s="276" t="s">
+      <c r="R23" s="285" t="s">
         <v>574</v>
       </c>
-      <c r="S23" s="276" t="s">
+      <c r="S23" s="285" t="s">
         <v>561</v>
       </c>
-      <c r="T23" s="275" t="s">
+      <c r="T23" s="284" t="s">
         <v>292</v>
       </c>
-      <c r="U23" s="275"/>
-      <c r="V23" s="275" t="s">
+      <c r="U23" s="284"/>
+      <c r="V23" s="284" t="s">
         <v>293</v>
       </c>
-      <c r="W23" s="275"/>
+      <c r="W23" s="284"/>
       <c r="X23" s="168" t="s">
         <v>462</v>
       </c>
@@ -38203,9 +38215,9 @@
       <c r="P24" s="170" t="s">
         <v>463</v>
       </c>
-      <c r="Q24" s="276"/>
-      <c r="R24" s="276"/>
-      <c r="S24" s="276"/>
+      <c r="Q24" s="285"/>
+      <c r="R24" s="285"/>
+      <c r="S24" s="285"/>
       <c r="T24" s="244" t="s">
         <v>463</v>
       </c>
@@ -66797,13 +66809,13 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="F1:AE32"/>
+  <dimension ref="F1:AR32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="18" max="18" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="6:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="6:44" x14ac:dyDescent="0.25">
       <c r="F1" s="4" t="s">
         <v>332</v>
       </c>
@@ -66811,12 +66823,12 @@
         <v>333</v>
       </c>
     </row>
-    <row r="2" spans="6:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="6:44" x14ac:dyDescent="0.25">
       <c r="G2" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="3" spans="6:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="6:44" x14ac:dyDescent="0.25">
       <c r="F3" t="s">
         <v>331</v>
       </c>
@@ -66830,7 +66842,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="4" spans="6:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="6:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F4">
         <v>400</v>
       </c>
@@ -66885,8 +66897,19 @@
       <c r="AE4" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="5" spans="6:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AH4" s="15"/>
+      <c r="AI4" s="15"/>
+      <c r="AJ4" s="15"/>
+      <c r="AK4" s="15"/>
+      <c r="AL4" s="15"/>
+      <c r="AM4" s="15"/>
+      <c r="AN4" s="15"/>
+      <c r="AO4" s="15"/>
+      <c r="AP4" s="15"/>
+      <c r="AQ4" s="15"/>
+      <c r="AR4" s="15"/>
+    </row>
+    <row r="5" spans="6:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F5">
         <v>500</v>
       </c>
@@ -66944,8 +66967,19 @@
       <c r="AE5" s="125">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="6:31" x14ac:dyDescent="0.25">
+      <c r="AH5" s="15"/>
+      <c r="AI5" s="15"/>
+      <c r="AJ5" s="15"/>
+      <c r="AK5" s="15"/>
+      <c r="AL5" s="15"/>
+      <c r="AM5" s="15"/>
+      <c r="AN5" s="15"/>
+      <c r="AO5" s="15"/>
+      <c r="AP5" s="15"/>
+      <c r="AQ5" s="15"/>
+      <c r="AR5" s="15"/>
+    </row>
+    <row r="6" spans="6:44" x14ac:dyDescent="0.25">
       <c r="F6">
         <v>600</v>
       </c>
@@ -67009,8 +67043,19 @@
       <c r="AE6" s="128">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="6:31" x14ac:dyDescent="0.25">
+      <c r="AH6" s="15"/>
+      <c r="AI6" s="15"/>
+      <c r="AJ6" s="15"/>
+      <c r="AK6" s="15"/>
+      <c r="AL6" s="15"/>
+      <c r="AM6" s="15"/>
+      <c r="AN6" s="15"/>
+      <c r="AO6" s="15"/>
+      <c r="AP6" s="15"/>
+      <c r="AQ6" s="15"/>
+      <c r="AR6" s="15"/>
+    </row>
+    <row r="7" spans="6:44" x14ac:dyDescent="0.25">
       <c r="F7">
         <v>700</v>
       </c>
@@ -67076,8 +67121,19 @@
       <c r="AE7" s="128">
         <v>8.5</v>
       </c>
-    </row>
-    <row r="8" spans="6:31" x14ac:dyDescent="0.25">
+      <c r="AH7" s="282"/>
+      <c r="AI7" s="282"/>
+      <c r="AJ7" s="15"/>
+      <c r="AK7" s="15"/>
+      <c r="AL7" s="15"/>
+      <c r="AM7" s="15"/>
+      <c r="AN7" s="15"/>
+      <c r="AO7" s="15"/>
+      <c r="AP7" s="15"/>
+      <c r="AQ7" s="15"/>
+      <c r="AR7" s="15"/>
+    </row>
+    <row r="8" spans="6:44" x14ac:dyDescent="0.25">
       <c r="R8" s="116">
         <v>40</v>
       </c>
@@ -67094,10 +67150,10 @@
         <v>19</v>
       </c>
       <c r="W8" s="113"/>
-      <c r="X8" t="s">
+      <c r="X8" s="276" t="s">
         <v>368</v>
       </c>
-      <c r="Y8">
+      <c r="Y8" s="10">
         <v>0</v>
       </c>
       <c r="AB8" s="134">
@@ -67113,8 +67169,19 @@
       <c r="AE8" s="128">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="6:31" x14ac:dyDescent="0.25">
+      <c r="AH8" s="136"/>
+      <c r="AI8" s="136"/>
+      <c r="AJ8" s="15"/>
+      <c r="AK8" s="15"/>
+      <c r="AL8" s="15"/>
+      <c r="AM8" s="15"/>
+      <c r="AN8" s="15"/>
+      <c r="AO8" s="15"/>
+      <c r="AP8" s="15"/>
+      <c r="AQ8" s="15"/>
+      <c r="AR8" s="15"/>
+    </row>
+    <row r="9" spans="6:44" x14ac:dyDescent="0.25">
       <c r="R9" s="116">
         <v>50</v>
       </c>
@@ -67131,10 +67198,10 @@
         <v>21</v>
       </c>
       <c r="W9" s="113"/>
-      <c r="X9" t="s">
+      <c r="X9" s="14" t="s">
         <v>331</v>
       </c>
-      <c r="Y9" s="136">
+      <c r="Y9" s="280">
         <v>0.16</v>
       </c>
       <c r="AB9" s="134">
@@ -67150,8 +67217,19 @@
       <c r="AE9" s="128">
         <v>11.5</v>
       </c>
-    </row>
-    <row r="10" spans="6:31" x14ac:dyDescent="0.25">
+      <c r="AH9" s="136"/>
+      <c r="AI9" s="136"/>
+      <c r="AJ9" s="15"/>
+      <c r="AK9" s="15"/>
+      <c r="AL9" s="15"/>
+      <c r="AM9" s="15"/>
+      <c r="AN9" s="15"/>
+      <c r="AO9" s="15"/>
+      <c r="AP9" s="15"/>
+      <c r="AQ9" s="15"/>
+      <c r="AR9" s="15"/>
+    </row>
+    <row r="10" spans="6:44" x14ac:dyDescent="0.25">
       <c r="R10" s="116">
         <v>60</v>
       </c>
@@ -67168,10 +67246,10 @@
         <v>23</v>
       </c>
       <c r="W10" s="113"/>
-      <c r="X10" t="s">
+      <c r="X10" s="278" t="s">
         <v>337</v>
       </c>
-      <c r="Y10">
+      <c r="Y10" s="281">
         <v>12.5</v>
       </c>
       <c r="AB10" s="135">
@@ -67187,8 +67265,19 @@
       <c r="AE10" s="131">
         <v>13</v>
       </c>
-    </row>
-    <row r="11" spans="6:31" x14ac:dyDescent="0.25">
+      <c r="AH10" s="136"/>
+      <c r="AI10" s="136"/>
+      <c r="AJ10" s="15"/>
+      <c r="AK10" s="15"/>
+      <c r="AL10" s="15"/>
+      <c r="AM10" s="15"/>
+      <c r="AN10" s="15"/>
+      <c r="AO10" s="15"/>
+      <c r="AP10" s="15"/>
+      <c r="AQ10" s="15"/>
+      <c r="AR10" s="15"/>
+    </row>
+    <row r="11" spans="6:44" x14ac:dyDescent="0.25">
       <c r="R11" s="116">
         <v>70</v>
       </c>
@@ -67220,8 +67309,19 @@
       <c r="AE11" s="125">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="6:31" x14ac:dyDescent="0.25">
+      <c r="AH11" s="136"/>
+      <c r="AI11" s="136"/>
+      <c r="AJ11" s="15"/>
+      <c r="AK11" s="15"/>
+      <c r="AL11" s="15"/>
+      <c r="AM11" s="15"/>
+      <c r="AN11" s="15"/>
+      <c r="AO11" s="15"/>
+      <c r="AP11" s="15"/>
+      <c r="AQ11" s="15"/>
+      <c r="AR11" s="15"/>
+    </row>
+    <row r="12" spans="6:44" x14ac:dyDescent="0.25">
       <c r="R12" s="117">
         <v>80</v>
       </c>
@@ -67236,6 +67336,12 @@
       </c>
       <c r="V12" s="132">
         <v>28</v>
+      </c>
+      <c r="X12" s="276" t="s">
+        <v>368</v>
+      </c>
+      <c r="Y12" s="10">
+        <v>0</v>
       </c>
       <c r="AB12" s="134">
         <v>40</v>
@@ -67250,8 +67356,25 @@
       <c r="AE12" s="128">
         <v>9.5</v>
       </c>
-    </row>
-    <row r="13" spans="6:31" x14ac:dyDescent="0.25">
+      <c r="AH12" s="136"/>
+      <c r="AI12" s="136"/>
+      <c r="AJ12" s="15"/>
+      <c r="AK12" s="15"/>
+      <c r="AL12" s="15"/>
+      <c r="AM12" s="15"/>
+      <c r="AN12" s="15"/>
+      <c r="AO12" s="15"/>
+      <c r="AP12" s="15"/>
+      <c r="AQ12" s="15"/>
+      <c r="AR12" s="15"/>
+    </row>
+    <row r="13" spans="6:44" x14ac:dyDescent="0.25">
+      <c r="X13" s="14" t="s">
+        <v>367</v>
+      </c>
+      <c r="Y13" s="277">
+        <v>0.46328995179259302</v>
+      </c>
       <c r="AB13" s="134">
         <v>50</v>
       </c>
@@ -67265,8 +67388,19 @@
       <c r="AE13" s="128">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="6:31" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="AH13" s="15"/>
+      <c r="AI13" s="15"/>
+      <c r="AJ13" s="15"/>
+      <c r="AK13" s="15"/>
+      <c r="AL13" s="15"/>
+      <c r="AM13" s="15"/>
+      <c r="AN13" s="15"/>
+      <c r="AO13" s="15"/>
+      <c r="AP13" s="15"/>
+      <c r="AQ13" s="15"/>
+      <c r="AR13" s="15"/>
+    </row>
+    <row r="14" spans="6:44" ht="15.75" x14ac:dyDescent="0.25">
       <c r="R14" s="140" t="s">
         <v>373</v>
       </c>
@@ -67274,6 +67408,13 @@
       <c r="T14" s="118"/>
       <c r="U14" s="118"/>
       <c r="V14" s="118"/>
+      <c r="X14" s="278" t="s">
+        <v>337</v>
+      </c>
+      <c r="Y14" s="279">
+        <f>0.0125625963867342*1000</f>
+        <v>12.562596386734201</v>
+      </c>
       <c r="AB14" s="134">
         <v>60</v>
       </c>
@@ -67287,8 +67428,19 @@
       <c r="AE14" s="128">
         <v>12.5</v>
       </c>
-    </row>
-    <row r="15" spans="6:31" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="AH14" s="15"/>
+      <c r="AI14" s="15"/>
+      <c r="AJ14" s="15"/>
+      <c r="AK14" s="15"/>
+      <c r="AL14" s="15"/>
+      <c r="AM14" s="15"/>
+      <c r="AN14" s="15"/>
+      <c r="AO14" s="15"/>
+      <c r="AP14" s="15"/>
+      <c r="AQ14" s="15"/>
+      <c r="AR14" s="15"/>
+    </row>
+    <row r="15" spans="6:44" ht="15.75" x14ac:dyDescent="0.25">
       <c r="R15" s="119" t="s">
         <v>336</v>
       </c>
@@ -67311,8 +67463,19 @@
       <c r="AE15" s="128">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="6:31" x14ac:dyDescent="0.25">
+      <c r="AH15" s="283"/>
+      <c r="AI15" s="283"/>
+      <c r="AJ15" s="283"/>
+      <c r="AK15" s="283"/>
+      <c r="AL15" s="283"/>
+      <c r="AM15" s="283"/>
+      <c r="AN15" s="15"/>
+      <c r="AO15" s="15"/>
+      <c r="AP15" s="15"/>
+      <c r="AQ15" s="15"/>
+      <c r="AR15" s="15"/>
+    </row>
+    <row r="16" spans="6:44" x14ac:dyDescent="0.25">
       <c r="R16" s="120" t="s">
         <v>123</v>
       </c>
@@ -67341,26 +67504,37 @@
       <c r="AE16" s="131">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="AH16" s="136"/>
+      <c r="AI16" s="136"/>
+      <c r="AJ16" s="136"/>
+      <c r="AK16" s="136"/>
+      <c r="AL16" s="136"/>
+      <c r="AM16" s="136"/>
+      <c r="AN16" s="15"/>
+      <c r="AO16" s="15"/>
+      <c r="AP16" s="15"/>
+      <c r="AQ16" s="15"/>
+      <c r="AR16" s="15"/>
+    </row>
+    <row r="17" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R17" s="114">
         <v>30</v>
       </c>
       <c r="S17" s="142">
-        <f t="shared" ref="S17:V22" si="2">($Y$8+$R17*$Y$9+S$16*$Y$10)/S7</f>
-        <v>0.79999999999999993</v>
+        <f>($Y$12+$R17^0.75*$Y$13+S$16*$Y$14)/S7</f>
+        <v>0.98978888297456324</v>
       </c>
       <c r="T17" s="143">
-        <f t="shared" si="2"/>
-        <v>0.99062499999999998</v>
+        <f t="shared" ref="T17:V17" si="2">($Y$12+$R17^0.75*$Y$13+T$16*$Y$14)/T7</f>
+        <v>1.1349227993163662</v>
       </c>
       <c r="U17" s="143">
         <f t="shared" si="2"/>
-        <v>1.0045454545454546</v>
+        <v>1.1109119537467711</v>
       </c>
       <c r="V17" s="144">
         <f t="shared" si="2"/>
-        <v>0.98857142857142866</v>
+        <v>1.0572188391189474</v>
       </c>
       <c r="AB17" s="133">
         <v>30</v>
@@ -67375,26 +67549,37 @@
       <c r="AE17" s="125">
         <v>11</v>
       </c>
-    </row>
-    <row r="18" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="AH17" s="136"/>
+      <c r="AI17" s="136"/>
+      <c r="AJ17" s="136"/>
+      <c r="AK17" s="136"/>
+      <c r="AL17" s="136"/>
+      <c r="AM17" s="136"/>
+      <c r="AN17" s="15"/>
+      <c r="AO17" s="15"/>
+      <c r="AP17" s="15"/>
+      <c r="AQ17" s="15"/>
+      <c r="AR17" s="15"/>
+    </row>
+    <row r="18" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R18" s="116">
         <v>40</v>
       </c>
       <c r="S18" s="145">
-        <f t="shared" si="2"/>
-        <v>0.91428571428571437</v>
+        <f t="shared" ref="S18:V18" si="3">($Y$12+$R18^0.75*$Y$13+S$16*$Y$14)/S8</f>
+        <v>1.0526883931215636</v>
       </c>
       <c r="T18" s="146">
-        <f>($Y$8+$R18*$Y$9+T$16*$Y$10)/T8</f>
-        <v>1.0026315789473685</v>
+        <f t="shared" si="3"/>
+        <v>1.1062597735299469</v>
       </c>
       <c r="U18" s="146">
-        <f t="shared" si="2"/>
-        <v>1.012</v>
+        <f t="shared" si="3"/>
+        <v>1.0920093556174435</v>
       </c>
       <c r="V18" s="147">
-        <f t="shared" si="2"/>
-        <v>0.99473684210526303</v>
+        <f t="shared" si="3"/>
+        <v>1.0490218493992181</v>
       </c>
       <c r="AB18" s="134">
         <v>40</v>
@@ -67409,26 +67594,37 @@
       <c r="AE18" s="128">
         <v>12.5</v>
       </c>
-    </row>
-    <row r="19" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="AH18" s="136"/>
+      <c r="AI18" s="136"/>
+      <c r="AJ18" s="136"/>
+      <c r="AK18" s="136"/>
+      <c r="AL18" s="136"/>
+      <c r="AM18" s="136"/>
+      <c r="AN18" s="15"/>
+      <c r="AO18" s="15"/>
+      <c r="AP18" s="15"/>
+      <c r="AQ18" s="15"/>
+      <c r="AR18" s="15"/>
+    </row>
+    <row r="19" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R19" s="116">
         <v>50</v>
       </c>
       <c r="S19" s="145">
-        <f t="shared" si="2"/>
-        <v>0.94117647058823528</v>
+        <f>($Y$12+$R19^0.75*$Y$13+S$16*$Y$14)/S9</f>
+        <v>1.0248527210041596</v>
       </c>
       <c r="T19" s="146">
-        <f t="shared" si="2"/>
-        <v>1.0113636363636365</v>
+        <f t="shared" ref="T19:V19" si="4">($Y$12+$R19^0.75*$Y$13+T$16*$Y$14)/T9</f>
+        <v>1.0774452022926277</v>
       </c>
       <c r="U19" s="146">
-        <f t="shared" si="2"/>
-        <v>1.0178571428571428</v>
+        <f t="shared" si="4"/>
+        <v>1.0708961658501754</v>
       </c>
       <c r="V19" s="147">
-        <f t="shared" si="2"/>
-        <v>0.97619047619047616</v>
+        <f t="shared" si="4"/>
+        <v>1.0130402150128361</v>
       </c>
       <c r="AB19" s="134">
         <v>50</v>
@@ -67443,26 +67639,37 @@
       <c r="AE19" s="128">
         <v>14</v>
       </c>
-    </row>
-    <row r="20" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="AH19" s="15"/>
+      <c r="AI19" s="15"/>
+      <c r="AJ19" s="15"/>
+      <c r="AK19" s="15"/>
+      <c r="AL19" s="15"/>
+      <c r="AM19" s="15"/>
+      <c r="AN19" s="15"/>
+      <c r="AO19" s="15"/>
+      <c r="AP19" s="15"/>
+      <c r="AQ19" s="15"/>
+      <c r="AR19" s="15"/>
+    </row>
+    <row r="20" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R20" s="116">
         <v>60</v>
       </c>
       <c r="S20" s="145">
-        <f t="shared" si="2"/>
-        <v>0.96</v>
+        <f t="shared" ref="S20:V20" si="5">($Y$12+$R20^0.75*$Y$13+S$16*$Y$14)/S10</f>
+        <v>0.99877190826154594</v>
       </c>
       <c r="T20" s="146">
-        <f t="shared" si="2"/>
-        <v>1.018</v>
+        <f t="shared" si="5"/>
+        <v>1.0502694543439208</v>
       </c>
       <c r="U20" s="146">
-        <f t="shared" si="2"/>
-        <v>1.0225806451612902</v>
+        <f t="shared" si="5"/>
+        <v>1.0496140178053264</v>
       </c>
       <c r="V20" s="147">
-        <f t="shared" si="2"/>
-        <v>0.96086956521739142</v>
+        <f t="shared" si="5"/>
+        <v>0.9804484986673766</v>
       </c>
       <c r="AB20" s="134">
         <v>60</v>
@@ -67477,26 +67684,37 @@
       <c r="AE20" s="128">
         <v>15.5</v>
       </c>
-    </row>
-    <row r="21" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="AH20" s="283"/>
+      <c r="AI20" s="283"/>
+      <c r="AJ20" s="283"/>
+      <c r="AK20" s="283"/>
+      <c r="AL20" s="283"/>
+      <c r="AM20" s="283"/>
+      <c r="AN20" s="283"/>
+      <c r="AO20" s="283"/>
+      <c r="AP20" s="283"/>
+      <c r="AQ20" s="15"/>
+      <c r="AR20" s="15"/>
+    </row>
+    <row r="21" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R21" s="116">
         <v>70</v>
       </c>
       <c r="S21" s="145">
-        <f t="shared" si="2"/>
-        <v>0.97391304347826091</v>
+        <f>($Y$12+$R21^0.75*$Y$13+S$16*$Y$14)/S11</f>
+        <v>0.97494153004629269</v>
       </c>
       <c r="T21" s="146">
-        <f t="shared" si="2"/>
-        <v>1.0232142857142859</v>
+        <f t="shared" ref="T21:V21" si="6">($Y$12+$R21^0.75*$Y$13+T$16*$Y$14)/T11</f>
+        <v>1.0251769065868512</v>
       </c>
       <c r="U21" s="146">
-        <f t="shared" si="2"/>
-        <v>0.99714285714285733</v>
+        <f t="shared" si="6"/>
+        <v>0.99960718793711234</v>
       </c>
       <c r="V21" s="147">
-        <f t="shared" si="2"/>
-        <v>0.94800000000000006</v>
+        <f t="shared" si="6"/>
+        <v>0.95097695929066273</v>
       </c>
       <c r="AB21" s="134">
         <v>70</v>
@@ -67511,26 +67729,37 @@
       <c r="AE21" s="128">
         <v>17.5</v>
       </c>
-    </row>
-    <row r="22" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="AH21" s="136"/>
+      <c r="AI21" s="136"/>
+      <c r="AJ21" s="136"/>
+      <c r="AK21" s="136"/>
+      <c r="AL21" s="136"/>
+      <c r="AM21" s="136"/>
+      <c r="AN21" s="136"/>
+      <c r="AO21" s="136"/>
+      <c r="AP21" s="136"/>
+      <c r="AQ21" s="15"/>
+      <c r="AR21" s="15"/>
+    </row>
+    <row r="22" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R22" s="117">
         <v>80</v>
       </c>
       <c r="S22" s="148">
-        <f t="shared" si="2"/>
-        <v>0.98461538461538467</v>
+        <f t="shared" ref="S22:V22" si="7">($Y$12+$R22^0.75*$Y$13+S$16*$Y$14)/S12</f>
+        <v>0.95329434970550908</v>
       </c>
       <c r="T22" s="149">
-        <f t="shared" si="2"/>
-        <v>0.99531250000000004</v>
+        <f t="shared" si="7"/>
+        <v>0.97084222767844797</v>
       </c>
       <c r="U22" s="149">
-        <f t="shared" si="2"/>
-        <v>0.97692307692307701</v>
+        <f t="shared" si="7"/>
+        <v>0.9576474225404471</v>
       </c>
       <c r="V22" s="150">
-        <f t="shared" si="2"/>
-        <v>0.90357142857142858</v>
+        <f t="shared" si="7"/>
+        <v>0.89126510474663634</v>
       </c>
       <c r="AB22" s="135">
         <v>80</v>
@@ -67545,8 +67774,19 @@
       <c r="AE22" s="131">
         <v>19.5</v>
       </c>
-    </row>
-    <row r="23" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="AH22" s="136"/>
+      <c r="AI22" s="136"/>
+      <c r="AJ22" s="136"/>
+      <c r="AK22" s="136"/>
+      <c r="AL22" s="136"/>
+      <c r="AM22" s="136"/>
+      <c r="AN22" s="136"/>
+      <c r="AO22" s="136"/>
+      <c r="AP22" s="136"/>
+      <c r="AQ22" s="15"/>
+      <c r="AR22" s="15"/>
+    </row>
+    <row r="23" spans="18:44" x14ac:dyDescent="0.25">
       <c r="AB23" s="133">
         <v>30</v>
       </c>
@@ -67560,8 +67800,19 @@
       <c r="AE23" s="125">
         <v>17.5</v>
       </c>
-    </row>
-    <row r="24" spans="18:31" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="AH23" s="136"/>
+      <c r="AI23" s="136"/>
+      <c r="AJ23" s="136"/>
+      <c r="AK23" s="136"/>
+      <c r="AL23" s="136"/>
+      <c r="AM23" s="136"/>
+      <c r="AN23" s="136"/>
+      <c r="AO23" s="136"/>
+      <c r="AP23" s="136"/>
+      <c r="AQ23" s="15"/>
+      <c r="AR23" s="15"/>
+    </row>
+    <row r="24" spans="18:44" ht="15.75" x14ac:dyDescent="0.25">
       <c r="R24" s="140" t="s">
         <v>372</v>
       </c>
@@ -67582,8 +67833,19 @@
       <c r="AE24" s="128">
         <v>19</v>
       </c>
-    </row>
-    <row r="25" spans="18:31" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="AH24" s="15"/>
+      <c r="AI24" s="15"/>
+      <c r="AJ24" s="15"/>
+      <c r="AK24" s="15"/>
+      <c r="AL24" s="15"/>
+      <c r="AM24" s="15"/>
+      <c r="AN24" s="15"/>
+      <c r="AO24" s="15"/>
+      <c r="AP24" s="15"/>
+      <c r="AQ24" s="15"/>
+      <c r="AR24" s="15"/>
+    </row>
+    <row r="25" spans="18:44" ht="15.75" x14ac:dyDescent="0.25">
       <c r="R25" s="119" t="s">
         <v>336</v>
       </c>
@@ -67606,8 +67868,19 @@
       <c r="AE25" s="128">
         <v>21</v>
       </c>
-    </row>
-    <row r="26" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="AH25" s="15"/>
+      <c r="AI25" s="15"/>
+      <c r="AJ25" s="15"/>
+      <c r="AK25" s="15"/>
+      <c r="AL25" s="15"/>
+      <c r="AM25" s="15"/>
+      <c r="AN25" s="15"/>
+      <c r="AO25" s="15"/>
+      <c r="AP25" s="15"/>
+      <c r="AQ25" s="15"/>
+      <c r="AR25" s="15"/>
+    </row>
+    <row r="26" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R26" s="120" t="s">
         <v>123</v>
       </c>
@@ -67636,8 +67909,19 @@
       <c r="AE26" s="128">
         <v>23</v>
       </c>
-    </row>
-    <row r="27" spans="18:31" x14ac:dyDescent="0.25">
+      <c r="AH26" s="15"/>
+      <c r="AI26" s="15"/>
+      <c r="AJ26" s="15"/>
+      <c r="AK26" s="15"/>
+      <c r="AL26" s="15"/>
+      <c r="AM26" s="15"/>
+      <c r="AN26" s="15"/>
+      <c r="AO26" s="15"/>
+      <c r="AP26" s="15"/>
+      <c r="AQ26" s="15"/>
+      <c r="AR26" s="15"/>
+    </row>
+    <row r="27" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R27" s="114">
         <v>30</v>
       </c>
@@ -67646,15 +67930,15 @@
         <v>1.0148066401910558</v>
       </c>
       <c r="T27" s="143">
-        <f t="shared" ref="T27:V27" si="3">(0.475*$R27^0.75 + T$26*$X$27)/T7</f>
+        <f t="shared" ref="T27:V27" si="8">(0.475*$R27^0.75 + T$26*$X$27)/T7</f>
         <v>1.1361049801432919</v>
       </c>
       <c r="U27" s="143">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>1.0989854401042123</v>
       </c>
       <c r="V27" s="144">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>1.0336479909226477</v>
       </c>
       <c r="X27">
@@ -67674,24 +67958,24 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="18:31" x14ac:dyDescent="0.25">
+    <row r="28" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R28" s="116">
         <v>40</v>
       </c>
       <c r="S28" s="145">
-        <f t="shared" ref="S28:V28" si="4">(0.475*$R28^0.75 + S$26*$X$27)/S8</f>
+        <f t="shared" ref="S28:V28" si="9">(0.475*$R28^0.75 + S$26*$X$27)/S8</f>
         <v>1.0792959890409974</v>
       </c>
       <c r="T28" s="146">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>1.1110602024512612</v>
       </c>
       <c r="U28" s="146">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>1.0844057538629586</v>
       </c>
       <c r="V28" s="147">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>1.0292143117519463</v>
       </c>
       <c r="X28">
@@ -67711,92 +67995,117 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="18:31" x14ac:dyDescent="0.25">
+    <row r="29" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R29" s="116">
         <v>50</v>
       </c>
       <c r="S29" s="145">
-        <f t="shared" ref="S29:V29" si="5">(0.475*$R29^0.75 + S$26*$X$27)/S9</f>
+        <f t="shared" ref="S29:V29" si="10">(0.475*$R29^0.75 + S$26*$X$27)/S9</f>
         <v>1.0507567465976686</v>
       </c>
       <c r="T29" s="146">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>1.0846756678254712</v>
       </c>
       <c r="U29" s="146">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>1.0665308818628703</v>
       </c>
       <c r="V29" s="147">
-        <f t="shared" si="5"/>
+        <f t="shared" si="10"/>
         <v>0.99673487362286584</v>
       </c>
     </row>
-    <row r="30" spans="18:31" x14ac:dyDescent="0.25">
+    <row r="30" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R30" s="116">
         <v>60</v>
       </c>
       <c r="S30" s="145">
-        <f t="shared" ref="S30:V30" si="6">(0.475*$R30^0.75 + S$26*$X$27)/S10</f>
+        <f t="shared" ref="S30:V30" si="11">(0.475*$R30^0.75 + S$26*$X$27)/S10</f>
         <v>1.0240167190947895</v>
       </c>
       <c r="T30" s="146">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v>1.0592133752758317</v>
       </c>
       <c r="U30" s="146">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v>1.0477527219966383</v>
       </c>
       <c r="V30" s="147">
-        <f t="shared" si="6"/>
+        <f t="shared" si="11"/>
         <v>0.966963790910778</v>
       </c>
     </row>
-    <row r="31" spans="18:31" x14ac:dyDescent="0.25">
+    <row r="31" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R31" s="116">
         <v>70</v>
       </c>
       <c r="S31" s="145">
-        <f t="shared" ref="S31:V31" si="7">(0.475*$R31^0.75 + S$26*$X$27)/S11</f>
+        <f t="shared" ref="S31:V31" si="12">(0.475*$R31^0.75 + S$26*$X$27)/S11</f>
         <v>0.99958400776909073</v>
       </c>
       <c r="T31" s="146">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>1.0353725778103244</v>
       </c>
       <c r="U31" s="146">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>0.99972663367683112</v>
       </c>
       <c r="V31" s="147">
-        <f t="shared" si="7"/>
+        <f t="shared" si="12"/>
         <v>0.9398086435737818</v>
       </c>
     </row>
-    <row r="32" spans="18:31" x14ac:dyDescent="0.25">
+    <row r="32" spans="18:44" x14ac:dyDescent="0.25">
       <c r="R32" s="117">
         <v>80</v>
       </c>
       <c r="S32" s="148">
-        <f t="shared" ref="S32:V32" si="8">(0.475*$R32^0.75 + S$26*$X$27)/S12</f>
+        <f t="shared" ref="S32:V32" si="13">(0.475*$R32^0.75 + S$26*$X$27)/S12</f>
         <v>0.9773896765040011</v>
       </c>
       <c r="T32" s="149">
-        <f t="shared" si="8"/>
+        <f t="shared" si="13"/>
         <v>0.98162911215950088</v>
       </c>
       <c r="U32" s="149">
-        <f t="shared" si="8"/>
+        <f t="shared" si="13"/>
         <v>0.95928542536164174</v>
       </c>
       <c r="V32" s="150">
-        <f t="shared" si="8"/>
+        <f t="shared" si="13"/>
         <v>0.88235949266257196</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="S17:V22">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0.9"/>
+        <cfvo type="num" val="1"/>
+        <cfvo type="num" val="1.1000000000000001"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S27:V32">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0.9"/>
+        <cfvo type="num" val="1"/>
+        <cfvo type="num" val="1.1000000000000001"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed unit for max_fat. Should be g/kg DM, was % of DM
</commit_message>
<xml_diff>
--- a/data/default/CattleHerd.xlsx
+++ b/data/default/CattleHerd.xlsx
@@ -145,7 +145,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5596" uniqueCount="689">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5596" uniqueCount="690">
   <si>
     <t>value</t>
   </si>
@@ -2215,6 +2215,9 @@
   <si>
     <t>Spörndly (2003)</t>
   </si>
+  <si>
+    <t>g/kg DM</t>
+  </si>
 </sst>
 </file>
 
@@ -3713,13 +3716,13 @@
     <xf numFmtId="14" fontId="51" fillId="37" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -21050,7 +21053,7 @@
       <c r="J229" s="158" t="s">
         <v>680</v>
       </c>
-      <c r="K229" s="311">
+      <c r="K229" s="309">
         <v>0</v>
       </c>
       <c r="L229" s="158" t="s">
@@ -21064,7 +21067,7 @@
       <c r="J230" s="158" t="s">
         <v>682</v>
       </c>
-      <c r="K230" s="311">
+      <c r="K230" s="309">
         <v>0</v>
       </c>
       <c r="L230" s="158" t="s">
@@ -21078,7 +21081,7 @@
       <c r="J231" s="158" t="s">
         <v>683</v>
       </c>
-      <c r="K231" s="311">
+      <c r="K231" s="309">
         <v>0</v>
       </c>
       <c r="L231" s="158" t="s">
@@ -21092,7 +21095,7 @@
       <c r="J232" s="158" t="s">
         <v>685</v>
       </c>
-      <c r="K232" s="311">
+      <c r="K232" s="309">
         <v>0</v>
       </c>
       <c r="L232" s="158" t="s">
@@ -21309,10 +21312,10 @@
         <v>687</v>
       </c>
       <c r="K249" s="2">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="L249" t="s">
-        <v>311</v>
+        <v>689</v>
       </c>
       <c r="N249" t="s">
         <v>688</v>
@@ -43002,23 +43005,23 @@
       <c r="N24" s="168"/>
       <c r="O24" s="168"/>
       <c r="P24" s="168"/>
-      <c r="Q24" s="310" t="s">
+      <c r="Q24" s="311" t="s">
         <v>563</v>
       </c>
-      <c r="R24" s="310" t="s">
+      <c r="R24" s="311" t="s">
         <v>564</v>
       </c>
-      <c r="S24" s="310" t="s">
+      <c r="S24" s="311" t="s">
         <v>551</v>
       </c>
-      <c r="T24" s="309" t="s">
+      <c r="T24" s="310" t="s">
         <v>290</v>
       </c>
-      <c r="U24" s="309"/>
-      <c r="V24" s="309" t="s">
+      <c r="U24" s="310"/>
+      <c r="V24" s="310" t="s">
         <v>291</v>
       </c>
-      <c r="W24" s="309"/>
+      <c r="W24" s="310"/>
       <c r="X24" s="167" t="s">
         <v>455</v>
       </c>
@@ -43043,9 +43046,9 @@
       <c r="P25" s="169" t="s">
         <v>456</v>
       </c>
-      <c r="Q25" s="310"/>
-      <c r="R25" s="310"/>
-      <c r="S25" s="310"/>
+      <c r="Q25" s="311"/>
+      <c r="R25" s="311"/>
+      <c r="S25" s="311"/>
       <c r="T25" s="243" t="s">
         <v>456</v>
       </c>

</xml_diff>

<commit_message>
Slight update of calving interval for beef cows
</commit_message>
<xml_diff>
--- a/data/default/CattleHerd.xlsx
+++ b/data/default/CattleHerd.xlsx
@@ -143,7 +143,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5616" uniqueCount="734">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5618" uniqueCount="735">
   <si>
     <t>value</t>
   </si>
@@ -2347,6 +2347,9 @@
   </si>
   <si>
     <t>% of LW</t>
+  </si>
+  <si>
+    <t>not applicable to dairy cows</t>
   </si>
 </sst>
 </file>
@@ -3866,14 +3869,14 @@
     <xf numFmtId="9" fontId="35" fillId="0" borderId="0" xfId="42" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -15619,6 +15622,9 @@
       <c r="L27" t="s">
         <v>4</v>
       </c>
+      <c r="M27" t="s">
+        <v>734</v>
+      </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
@@ -15840,18 +15846,22 @@
       <c r="J39" t="s">
         <v>3</v>
       </c>
-      <c r="K39">
-        <v>12.7</v>
+      <c r="K39" s="13">
+        <f>(1291*12.4 + 3095*12.5 + 2319*12.5 + 1051*12.7 + 1624*12.6) / (1291 + 3095 + 2319 + 1051 + 1624)</f>
+        <v>12.525959488272919</v>
       </c>
       <c r="L39" t="s">
         <v>4</v>
       </c>
+      <c r="M39" t="s">
+        <v>720</v>
+      </c>
       <c r="N39" t="s">
         <v>719</v>
       </c>
       <c r="O39" s="318">
         <f>(12/K39)*(1*(1-K44/100)+2*K44/100)*(1-K45/100)</f>
-        <v>0.96237372896491069</v>
+        <v>0.97574532069156117</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
@@ -16448,7 +16458,7 @@
       <c r="M64" s="109" t="s">
         <v>616</v>
       </c>
-      <c r="O64" s="321">
+      <c r="O64" s="319">
         <f>O63</f>
         <v>0.515625</v>
       </c>
@@ -16772,7 +16782,7 @@
       <c r="M75" s="109" t="s">
         <v>616</v>
       </c>
-      <c r="O75" s="321">
+      <c r="O75" s="319">
         <f>O74</f>
         <v>0.5625</v>
       </c>
@@ -19183,7 +19193,7 @@
       <c r="N185" s="255" t="s">
         <v>658</v>
       </c>
-      <c r="O185" s="322">
+      <c r="O185" s="320">
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
@@ -19208,7 +19218,7 @@
         <v>660</v>
       </c>
       <c r="N186" s="255"/>
-      <c r="O186" s="322">
+      <c r="O186" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19232,7 +19242,7 @@
       <c r="M187" t="s">
         <v>660</v>
       </c>
-      <c r="O187" s="322">
+      <c r="O187" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19256,7 +19266,7 @@
       <c r="M188" t="s">
         <v>660</v>
       </c>
-      <c r="O188" s="322">
+      <c r="O188" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19280,7 +19290,7 @@
       <c r="M189" t="s">
         <v>660</v>
       </c>
-      <c r="O189" s="322">
+      <c r="O189" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19304,7 +19314,7 @@
       <c r="M190" t="s">
         <v>660</v>
       </c>
-      <c r="O190" s="322">
+      <c r="O190" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19328,7 +19338,7 @@
       <c r="M191" t="s">
         <v>660</v>
       </c>
-      <c r="O191" s="322">
+      <c r="O191" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19352,7 +19362,7 @@
       <c r="M192" t="s">
         <v>660</v>
       </c>
-      <c r="O192" s="322">
+      <c r="O192" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19376,7 +19386,7 @@
       <c r="M193" t="s">
         <v>660</v>
       </c>
-      <c r="O193" s="322">
+      <c r="O193" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19400,7 +19410,7 @@
       <c r="M194" t="s">
         <v>660</v>
       </c>
-      <c r="O194" s="322">
+      <c r="O194" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19424,7 +19434,7 @@
       <c r="M195" t="s">
         <v>660</v>
       </c>
-      <c r="O195" s="322">
+      <c r="O195" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -19448,7 +19458,7 @@
       <c r="M196" t="s">
         <v>660</v>
       </c>
-      <c r="O196" s="322">
+      <c r="O196" s="320">
         <v>0.03</v>
       </c>
     </row>
@@ -46068,23 +46078,23 @@
       <c r="N24" s="166"/>
       <c r="O24" s="166"/>
       <c r="P24" s="166"/>
-      <c r="Q24" s="320" t="s">
+      <c r="Q24" s="322" t="s">
         <v>560</v>
       </c>
-      <c r="R24" s="320" t="s">
+      <c r="R24" s="322" t="s">
         <v>561</v>
       </c>
-      <c r="S24" s="320" t="s">
+      <c r="S24" s="322" t="s">
         <v>548</v>
       </c>
-      <c r="T24" s="319" t="s">
+      <c r="T24" s="321" t="s">
         <v>287</v>
       </c>
-      <c r="U24" s="319"/>
-      <c r="V24" s="319" t="s">
+      <c r="U24" s="321"/>
+      <c r="V24" s="321" t="s">
         <v>288</v>
       </c>
-      <c r="W24" s="319"/>
+      <c r="W24" s="321"/>
       <c r="X24" s="165" t="s">
         <v>452</v>
       </c>
@@ -46129,9 +46139,9 @@
       <c r="P25" s="167" t="s">
         <v>453</v>
       </c>
-      <c r="Q25" s="320"/>
-      <c r="R25" s="320"/>
-      <c r="S25" s="320"/>
+      <c r="Q25" s="322"/>
+      <c r="R25" s="322"/>
+      <c r="S25" s="322"/>
       <c r="T25" s="241" t="s">
         <v>453</v>
       </c>

</xml_diff>